<commit_message>
Sprint 5: Remove RHI from holdings + auto-bust cache on file changes
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81FBE358-4532-464D-9E21-BC0C3B101201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{81FBE358-4532-464D-9E21-BC0C3B101201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AF332D8-4926-4429-8E17-95160E5D6428}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{182CA602-8141-4465-A9BC-B64C31C4A0CA}"/>
   </bookViews>
@@ -19,12 +19,25 @@
     <sheet name="OR" sheetId="4" r:id="rId4"/>
     <sheet name="DCP" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="1">
   <si>
     <t>Hughes, Robert (25208165, Individual)</t>
   </si>
@@ -890,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF4E0D3B-C480-43DD-AB9B-4533E533D134}">
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -982,7 +995,7 @@
         <v>46085</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B38" si="0">"*Quality Dividend Strategy (*QDG)"</f>
+        <f t="shared" ref="B2:B37" si="0">"*Quality Dividend Strategy (*QDG)"</f>
         <v>*Quality Dividend Strategy (*QDG)</v>
       </c>
       <c r="C2" s="2">
@@ -1857,7 +1870,7 @@
         <v>McCormick &amp; Co.</v>
       </c>
       <c r="G18">
-        <v>812</v>
+        <v>1075</v>
       </c>
       <c r="H18" s="1">
         <v>46014</v>
@@ -2480,48 +2493,49 @@
         <v>*Quality Dividend Strategy (*QDG)</v>
       </c>
       <c r="C30" s="2">
-        <v>8.6999999999999994E-3</v>
+        <v>1.77E-2</v>
       </c>
       <c r="D30" t="str">
-        <f>"RHI"</f>
-        <v>RHI</v>
-      </c>
-      <c r="E30">
-        <v>770323103</v>
+        <f>"TROW"</f>
+        <v>TROW</v>
+      </c>
+      <c r="E30" t="str">
+        <f>"74144T108"</f>
+        <v>74144T108</v>
       </c>
       <c r="F30" t="str">
-        <f>"Robert Half International"</f>
-        <v>Robert Half International</v>
+        <f>"T. Rowe Price"</f>
+        <v>T. Rowe Price</v>
       </c>
       <c r="G30">
-        <v>794</v>
+        <v>426</v>
       </c>
       <c r="H30" s="1">
-        <v>45588</v>
+        <v>44929</v>
       </c>
       <c r="I30" s="3">
-        <v>19310.080000000002</v>
+        <v>39187.74</v>
       </c>
       <c r="J30">
-        <v>24.32</v>
+        <v>91.99</v>
       </c>
       <c r="K30">
-        <v>43.37</v>
+        <v>111.82</v>
       </c>
       <c r="L30" s="3">
-        <v>34434.269999999997</v>
+        <v>47635.040000000001</v>
       </c>
       <c r="M30" s="3">
-        <v>1873.84</v>
+        <v>2215.1999999999998</v>
       </c>
       <c r="N30" s="3">
-        <v>3654.83</v>
+        <v>6052.14</v>
       </c>
       <c r="O30" s="2">
-        <v>5.4399999999999997E-2</v>
+        <v>4.65E-2</v>
       </c>
       <c r="P30" s="2">
-        <v>9.7000000000000003E-2</v>
+        <v>5.6500000000000002E-2</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
@@ -2533,49 +2547,48 @@
         <v>*Quality Dividend Strategy (*QDG)</v>
       </c>
       <c r="C31" s="2">
-        <v>1.77E-2</v>
+        <v>2.7400000000000001E-2</v>
       </c>
       <c r="D31" t="str">
-        <f>"TROW"</f>
-        <v>TROW</v>
-      </c>
-      <c r="E31" t="str">
-        <f>"74144T108"</f>
-        <v>74144T108</v>
+        <f>"TXN"</f>
+        <v>TXN</v>
+      </c>
+      <c r="E31">
+        <v>882508104</v>
       </c>
       <c r="F31" t="str">
-        <f>"T. Rowe Price"</f>
-        <v>T. Rowe Price</v>
+        <f>"Texas Instruments"</f>
+        <v>Texas Instruments</v>
       </c>
       <c r="G31">
-        <v>426</v>
+        <v>299</v>
       </c>
       <c r="H31" s="1">
-        <v>44929</v>
+        <v>41079</v>
       </c>
       <c r="I31" s="3">
-        <v>39187.74</v>
+        <v>60514.61</v>
       </c>
       <c r="J31">
-        <v>91.99</v>
+        <v>202.39</v>
       </c>
       <c r="K31">
-        <v>111.82</v>
+        <v>50.62</v>
       </c>
       <c r="L31" s="3">
-        <v>47635.040000000001</v>
+        <v>15136.68</v>
       </c>
       <c r="M31" s="3">
-        <v>2215.1999999999998</v>
+        <v>1698.32</v>
       </c>
       <c r="N31" s="3">
-        <v>6052.14</v>
+        <v>13958.55</v>
       </c>
       <c r="O31" s="2">
-        <v>4.65E-2</v>
+        <v>0.11219999999999999</v>
       </c>
       <c r="P31" s="2">
-        <v>5.6500000000000002E-2</v>
+        <v>2.81E-2</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
@@ -2587,48 +2600,50 @@
         <v>*Quality Dividend Strategy (*QDG)</v>
       </c>
       <c r="C32" s="2">
-        <v>2.7400000000000001E-2</v>
+        <v>1.9300000000000001E-2</v>
       </c>
       <c r="D32" t="str">
-        <f>"TXN"</f>
-        <v>TXN</v>
-      </c>
-      <c r="E32">
-        <v>882508104</v>
+        <f>"TTE"</f>
+        <v>TTE</v>
+      </c>
+      <c r="E32" t="str">
+        <f>"F92124100"</f>
+        <v>F92124100</v>
       </c>
       <c r="F32" t="str">
-        <f>"Texas Instruments"</f>
-        <v>Texas Instruments</v>
+        <f>"Total SA"</f>
+        <v>Total SA</v>
       </c>
       <c r="G32">
-        <v>299</v>
+        <v>556</v>
       </c>
       <c r="H32" s="1">
-        <v>41079</v>
+        <v>43874</v>
       </c>
       <c r="I32" s="3">
-        <v>60514.61</v>
+        <v>42767.519999999997</v>
       </c>
       <c r="J32">
-        <v>202.39</v>
+        <v>76.92</v>
       </c>
       <c r="K32">
-        <v>50.62</v>
+        <v>49.15</v>
       </c>
       <c r="L32" s="3">
-        <v>15136.68</v>
-      </c>
-      <c r="M32" s="3">
-        <v>1698.32</v>
+        <v>27327.39</v>
+      </c>
+      <c r="M32">
+        <v>0</v>
       </c>
       <c r="N32" s="3">
-        <v>13958.55</v>
-      </c>
-      <c r="O32" s="2">
-        <v>0.11219999999999999</v>
+        <v>9119.24</v>
+      </c>
+      <c r="O32" t="str">
+        <f>""</f>
+        <v/>
       </c>
       <c r="P32" s="2">
-        <v>2.81E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
@@ -2640,320 +2655,265 @@
         <v>*Quality Dividend Strategy (*QDG)</v>
       </c>
       <c r="C33" s="2">
-        <v>1.9300000000000001E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="D33" t="str">
-        <f>"TTE"</f>
-        <v>TTE</v>
-      </c>
-      <c r="E33" t="str">
-        <f>"F92124100"</f>
-        <v>F92124100</v>
+        <f>"UL"</f>
+        <v>UL</v>
+      </c>
+      <c r="E33">
+        <v>904767803</v>
       </c>
       <c r="F33" t="str">
-        <f>"Total SA"</f>
-        <v>Total SA</v>
+        <f>"Unilever PLC"</f>
+        <v>Unilever PLC</v>
       </c>
       <c r="G33">
-        <v>556</v>
+        <v>898</v>
       </c>
       <c r="H33" s="1">
-        <v>43874</v>
+        <v>43889</v>
       </c>
       <c r="I33" s="3">
-        <v>42767.519999999997</v>
+        <v>62024.86</v>
       </c>
       <c r="J33">
-        <v>76.92</v>
+        <v>69.069999999999993</v>
       </c>
       <c r="K33">
-        <v>49.15</v>
+        <v>58.12</v>
       </c>
       <c r="L33" s="3">
-        <v>27327.39</v>
-      </c>
-      <c r="M33">
-        <v>0</v>
+        <v>52191.45</v>
+      </c>
+      <c r="M33" s="3">
+        <v>2062.9499999999998</v>
       </c>
       <c r="N33" s="3">
-        <v>9119.24</v>
-      </c>
-      <c r="O33" t="str">
+        <v>11627.82</v>
+      </c>
+      <c r="O33" s="2">
+        <v>3.95E-2</v>
+      </c>
+      <c r="P33" s="2">
+        <v>3.3300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>*Quality Dividend Strategy (*QDG)</v>
+      </c>
+      <c r="C34" s="2">
+        <v>2.5700000000000001E-2</v>
+      </c>
+      <c r="D34" t="str">
+        <f>"UNP"</f>
+        <v>UNP</v>
+      </c>
+      <c r="E34">
+        <v>907818108</v>
+      </c>
+      <c r="F34" t="str">
+        <f>"Union Pacific"</f>
+        <v>Union Pacific</v>
+      </c>
+      <c r="G34">
+        <v>213</v>
+      </c>
+      <c r="H34" s="1">
+        <v>45092</v>
+      </c>
+      <c r="I34" s="3">
+        <v>56807.1</v>
+      </c>
+      <c r="J34">
+        <v>266.7</v>
+      </c>
+      <c r="K34">
+        <v>211.24</v>
+      </c>
+      <c r="L34" s="3">
+        <v>44993.19</v>
+      </c>
+      <c r="M34" s="3">
+        <v>1175.76</v>
+      </c>
+      <c r="N34" s="3">
+        <v>2264.04</v>
+      </c>
+      <c r="O34" s="2">
+        <v>2.6100000000000002E-2</v>
+      </c>
+      <c r="P34" s="2">
+        <v>2.07E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>*Quality Dividend Strategy (*QDG)</v>
+      </c>
+      <c r="C35" s="2">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="D35" t="str">
+        <f>"UPS"</f>
+        <v>UPS</v>
+      </c>
+      <c r="E35">
+        <v>911312106</v>
+      </c>
+      <c r="F35" t="str">
+        <f>"United Parcel Service"</f>
+        <v>United Parcel Service</v>
+      </c>
+      <c r="G35">
+        <v>405</v>
+      </c>
+      <c r="H35" s="1">
+        <v>45470</v>
+      </c>
+      <c r="I35" s="3">
+        <v>44752.5</v>
+      </c>
+      <c r="J35">
+        <v>110.5</v>
+      </c>
+      <c r="K35">
+        <v>103.25</v>
+      </c>
+      <c r="L35" s="3">
+        <v>41815.78</v>
+      </c>
+      <c r="M35" s="3">
+        <v>2656.8</v>
+      </c>
+      <c r="N35" s="3">
+        <v>11284.9</v>
+      </c>
+      <c r="O35" s="2">
+        <v>6.3500000000000001E-2</v>
+      </c>
+      <c r="P35" s="2">
+        <v>5.9400000000000001E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>*Quality Dividend Strategy (*QDG)</v>
+      </c>
+      <c r="C36" s="2">
+        <v>2.1299999999999999E-2</v>
+      </c>
+      <c r="D36" t="str">
+        <f>"VZ"</f>
+        <v>VZ</v>
+      </c>
+      <c r="E36" t="str">
+        <f>"92343V104"</f>
+        <v>92343V104</v>
+      </c>
+      <c r="F36" t="str">
+        <f>"Verizon"</f>
+        <v>Verizon</v>
+      </c>
+      <c r="G36">
+        <v>920</v>
+      </c>
+      <c r="H36" s="1">
+        <v>42241</v>
+      </c>
+      <c r="I36" s="3">
+        <v>47104</v>
+      </c>
+      <c r="J36">
+        <v>51.2</v>
+      </c>
+      <c r="K36">
+        <v>46.89</v>
+      </c>
+      <c r="L36" s="3">
+        <v>43136.03</v>
+      </c>
+      <c r="M36" s="3">
+        <v>2603.6</v>
+      </c>
+      <c r="N36" s="3">
+        <v>24861.360000000001</v>
+      </c>
+      <c r="O36" s="2">
+        <v>6.0400000000000002E-2</v>
+      </c>
+      <c r="P36" s="2">
+        <v>5.5300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>*Quality Dividend Strategy (*QDG)</v>
+      </c>
+      <c r="C37" s="2">
+        <v>8.6599999999999996E-2</v>
+      </c>
+      <c r="D37" t="str">
+        <f>"CASH"</f>
+        <v>CASH</v>
+      </c>
+      <c r="E37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="P33" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B34" t="str">
-        <f t="shared" si="0"/>
-        <v>*Quality Dividend Strategy (*QDG)</v>
-      </c>
-      <c r="C34" s="2">
-        <v>2.81E-2</v>
-      </c>
-      <c r="D34" t="str">
-        <f>"UL"</f>
-        <v>UL</v>
-      </c>
-      <c r="E34">
-        <v>904767803</v>
-      </c>
-      <c r="F34" t="str">
-        <f>"Unilever PLC"</f>
-        <v>Unilever PLC</v>
-      </c>
-      <c r="G34">
-        <v>898</v>
-      </c>
-      <c r="H34" s="1">
-        <v>43889</v>
-      </c>
-      <c r="I34" s="3">
-        <v>62024.86</v>
-      </c>
-      <c r="J34">
-        <v>69.069999999999993</v>
-      </c>
-      <c r="K34">
-        <v>58.12</v>
-      </c>
-      <c r="L34" s="3">
-        <v>52191.45</v>
-      </c>
-      <c r="M34" s="3">
-        <v>2062.9499999999998</v>
-      </c>
-      <c r="N34" s="3">
-        <v>11627.82</v>
-      </c>
-      <c r="O34" s="2">
-        <v>3.95E-2</v>
-      </c>
-      <c r="P34" s="2">
-        <v>3.3300000000000003E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B35" t="str">
-        <f t="shared" si="0"/>
-        <v>*Quality Dividend Strategy (*QDG)</v>
-      </c>
-      <c r="C35" s="2">
-        <v>2.5700000000000001E-2</v>
-      </c>
-      <c r="D35" t="str">
-        <f>"UNP"</f>
-        <v>UNP</v>
-      </c>
-      <c r="E35">
-        <v>907818108</v>
-      </c>
-      <c r="F35" t="str">
-        <f>"Union Pacific"</f>
-        <v>Union Pacific</v>
-      </c>
-      <c r="G35">
-        <v>213</v>
-      </c>
-      <c r="H35" s="1">
-        <v>45092</v>
-      </c>
-      <c r="I35" s="3">
-        <v>56807.1</v>
-      </c>
-      <c r="J35">
-        <v>266.7</v>
-      </c>
-      <c r="K35">
-        <v>211.24</v>
-      </c>
-      <c r="L35" s="3">
-        <v>44993.19</v>
-      </c>
-      <c r="M35" s="3">
-        <v>1175.76</v>
-      </c>
-      <c r="N35" s="3">
-        <v>2264.04</v>
-      </c>
-      <c r="O35" s="2">
-        <v>2.6100000000000002E-2</v>
-      </c>
-      <c r="P35" s="2">
-        <v>2.07E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B36" t="str">
-        <f t="shared" si="0"/>
-        <v>*Quality Dividend Strategy (*QDG)</v>
-      </c>
-      <c r="C36" s="2">
-        <v>2.0199999999999999E-2</v>
-      </c>
-      <c r="D36" t="str">
-        <f>"UPS"</f>
-        <v>UPS</v>
-      </c>
-      <c r="E36">
-        <v>911312106</v>
-      </c>
-      <c r="F36" t="str">
-        <f>"United Parcel Service"</f>
-        <v>United Parcel Service</v>
-      </c>
-      <c r="G36">
-        <v>405</v>
-      </c>
-      <c r="H36" s="1">
-        <v>45470</v>
-      </c>
-      <c r="I36" s="3">
-        <v>44752.5</v>
-      </c>
-      <c r="J36">
-        <v>110.5</v>
-      </c>
-      <c r="K36">
-        <v>103.25</v>
-      </c>
-      <c r="L36" s="3">
-        <v>41815.78</v>
-      </c>
-      <c r="M36" s="3">
-        <v>2656.8</v>
-      </c>
-      <c r="N36" s="3">
-        <v>11284.9</v>
-      </c>
-      <c r="O36" s="2">
-        <v>6.3500000000000001E-2</v>
-      </c>
-      <c r="P36" s="2">
-        <v>5.9400000000000001E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B37" t="str">
-        <f t="shared" si="0"/>
-        <v>*Quality Dividend Strategy (*QDG)</v>
-      </c>
-      <c r="C37" s="2">
-        <v>2.1299999999999999E-2</v>
-      </c>
-      <c r="D37" t="str">
-        <f>"VZ"</f>
-        <v>VZ</v>
-      </c>
-      <c r="E37" t="str">
-        <f>"92343V104"</f>
-        <v>92343V104</v>
-      </c>
       <c r="F37" t="str">
-        <f>"Verizon"</f>
-        <v>Verizon</v>
-      </c>
-      <c r="G37">
-        <v>920</v>
-      </c>
-      <c r="H37" s="1">
-        <v>42241</v>
-      </c>
-      <c r="I37" s="3">
-        <v>47104</v>
-      </c>
-      <c r="J37">
-        <v>51.2</v>
-      </c>
-      <c r="K37">
-        <v>46.89</v>
-      </c>
-      <c r="L37" s="3">
-        <v>43136.03</v>
-      </c>
-      <c r="M37" s="3">
-        <v>2603.6</v>
-      </c>
-      <c r="N37" s="3">
-        <v>24861.360000000001</v>
-      </c>
-      <c r="O37" s="2">
-        <v>6.0400000000000002E-2</v>
-      </c>
-      <c r="P37" s="2">
-        <v>5.5300000000000002E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B38" t="str">
-        <f t="shared" si="0"/>
-        <v>*Quality Dividend Strategy (*QDG)</v>
-      </c>
-      <c r="C38" s="2">
-        <v>8.6599999999999996E-2</v>
-      </c>
-      <c r="D38" t="str">
-        <f>"CASH"</f>
-        <v>CASH</v>
-      </c>
-      <c r="E38" t="str">
+        <f>"Cash"</f>
+        <v>Cash</v>
+      </c>
+      <c r="G37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F38" t="str">
-        <f>"Cash"</f>
-        <v>Cash</v>
-      </c>
-      <c r="G38" t="str">
+      <c r="H37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="H38" t="str">
+      <c r="I37" s="3">
+        <v>195988.46</v>
+      </c>
+      <c r="J37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="I38" s="3">
-        <v>191434.61</v>
-      </c>
-      <c r="J38" t="str">
+      <c r="K37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="K38" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="L38" s="3">
-        <v>191434.61</v>
-      </c>
-      <c r="M38" s="3">
+      <c r="L37" s="3">
+        <v>195988.46</v>
+      </c>
+      <c r="M37" s="3">
         <v>1914.35</v>
       </c>
-      <c r="N38">
+      <c r="N37">
         <v>0</v>
       </c>
-      <c r="O38" s="2">
+      <c r="O37" s="2">
         <v>0.01</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P37" s="2">
         <v>0.01</v>
       </c>
     </row>
@@ -2964,7 +2924,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85A93AE2-CF7B-4A2C-B776-1476DCA65D14}">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -3056,7 +3016,7 @@
         <v>46085</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" ref="B2:B25" si="0">"*Quality SMID Dividend Strategy (*SMID)"</f>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C2" s="2">
@@ -3110,7 +3070,7 @@
         <v>46085</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C3" s="2">
@@ -3164,7 +3124,7 @@
         <v>46085</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C4" s="2">
@@ -3218,7 +3178,7 @@
         <v>46085</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C5" s="2">
@@ -3272,7 +3232,7 @@
         <v>46085</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C6" s="2">
@@ -3325,7 +3285,7 @@
         <v>46085</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C7" s="2">
@@ -3378,7 +3338,7 @@
         <v>46085</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C8" s="2">
@@ -3432,7 +3392,7 @@
         <v>46085</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C9" s="2">
@@ -3485,7 +3445,7 @@
         <v>46085</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C10" s="2">
@@ -3538,7 +3498,7 @@
         <v>46085</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C11" s="2">
@@ -3591,7 +3551,7 @@
         <v>46085</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C12" s="2">
@@ -3644,7 +3604,7 @@
         <v>46085</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C13" s="2">
@@ -3697,7 +3657,7 @@
         <v>46085</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C14" s="2">
@@ -3750,7 +3710,7 @@
         <v>46085</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C15" s="2">
@@ -3803,7 +3763,7 @@
         <v>46085</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C16" s="2">
@@ -3856,7 +3816,7 @@
         <v>46085</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C17" s="2">
@@ -3909,7 +3869,7 @@
         <v>46085</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C18" s="2">
@@ -3962,7 +3922,7 @@
         <v>46085</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C19" s="2">
@@ -4016,7 +3976,7 @@
         <v>46085</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C20" s="2">
@@ -4070,7 +4030,7 @@
         <v>46085</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C21" s="2">
@@ -4123,52 +4083,52 @@
         <v>46085</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C22" s="2">
-        <v>1.4500000000000001E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="D22" t="str">
-        <f>"RHI"</f>
-        <v>RHI</v>
+        <f>"SNA"</f>
+        <v>SNA</v>
       </c>
       <c r="E22">
-        <v>770323103</v>
+        <v>833034101</v>
       </c>
       <c r="F22" t="str">
-        <f>"Robert Half International"</f>
-        <v>Robert Half International</v>
-      </c>
-      <c r="G22" s="3">
-        <v>1516</v>
+        <f>"Snap-On"</f>
+        <v>Snap-On</v>
+      </c>
+      <c r="G22">
+        <v>215</v>
       </c>
       <c r="H22" s="1">
-        <v>44985</v>
+        <v>43805</v>
       </c>
       <c r="I22" s="3">
-        <v>36869.120000000003</v>
+        <v>82452.5</v>
       </c>
       <c r="J22">
-        <v>24.32</v>
+        <v>383.5</v>
       </c>
       <c r="K22">
-        <v>44.26</v>
+        <v>151.1</v>
       </c>
       <c r="L22" s="3">
-        <v>67103.53</v>
+        <v>32486.27</v>
       </c>
       <c r="M22" s="3">
-        <v>3577.76</v>
+        <v>2098.4</v>
       </c>
       <c r="N22" s="3">
-        <v>15279.5</v>
+        <v>11201.02</v>
       </c>
       <c r="O22" s="2">
-        <v>5.33E-2</v>
+        <v>6.4600000000000005E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>9.7000000000000003E-2</v>
+        <v>2.5399999999999999E-2</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
@@ -4176,52 +4136,52 @@
         <v>46085</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C23" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="D23" t="str">
-        <f>"SNA"</f>
-        <v>SNA</v>
+        <f>"SWK"</f>
+        <v>SWK</v>
       </c>
       <c r="E23">
-        <v>833034101</v>
+        <v>854502101</v>
       </c>
       <c r="F23" t="str">
-        <f>"Snap-On"</f>
-        <v>Snap-On</v>
+        <f>"Stanley Black &amp; Decker"</f>
+        <v>Stanley Black &amp; Decker</v>
       </c>
       <c r="G23">
-        <v>215</v>
+        <v>910</v>
       </c>
       <c r="H23" s="1">
-        <v>43805</v>
+        <v>45442</v>
       </c>
       <c r="I23" s="3">
-        <v>82452.5</v>
+        <v>72599.8</v>
       </c>
       <c r="J23">
-        <v>383.5</v>
+        <v>79.78</v>
       </c>
       <c r="K23">
-        <v>151.1</v>
+        <v>84.37</v>
       </c>
       <c r="L23" s="3">
-        <v>32486.27</v>
+        <v>76777.919999999998</v>
       </c>
       <c r="M23" s="3">
-        <v>2098.4</v>
+        <v>3021.2</v>
       </c>
       <c r="N23" s="3">
-        <v>11201.02</v>
+        <v>4519.55</v>
       </c>
       <c r="O23" s="2">
-        <v>6.4600000000000005E-2</v>
+        <v>3.9300000000000002E-2</v>
       </c>
       <c r="P23" s="2">
-        <v>2.5399999999999999E-2</v>
+        <v>4.1599999999999998E-2</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
@@ -4229,52 +4189,53 @@
         <v>46085</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C24" s="2">
-        <v>2.8500000000000001E-2</v>
+        <v>2.7300000000000001E-2</v>
       </c>
       <c r="D24" t="str">
-        <f>"SWK"</f>
-        <v>SWK</v>
-      </c>
-      <c r="E24">
-        <v>854502101</v>
+        <f>"TROW"</f>
+        <v>TROW</v>
+      </c>
+      <c r="E24" t="str">
+        <f>"74144T108"</f>
+        <v>74144T108</v>
       </c>
       <c r="F24" t="str">
-        <f>"Stanley Black &amp; Decker"</f>
-        <v>Stanley Black &amp; Decker</v>
+        <f>"T. Rowe Price"</f>
+        <v>T. Rowe Price</v>
       </c>
       <c r="G24">
-        <v>910</v>
+        <v>756</v>
       </c>
       <c r="H24" s="1">
-        <v>45442</v>
+        <v>45700</v>
       </c>
       <c r="I24" s="3">
-        <v>72599.8</v>
+        <v>69544.44</v>
       </c>
       <c r="J24">
-        <v>79.78</v>
+        <v>91.99</v>
       </c>
       <c r="K24">
-        <v>84.37</v>
+        <v>106.27</v>
       </c>
       <c r="L24" s="3">
-        <v>76777.919999999998</v>
+        <v>80343.740000000005</v>
       </c>
       <c r="M24" s="3">
-        <v>3021.2</v>
+        <v>3931.2</v>
       </c>
       <c r="N24" s="3">
-        <v>4519.55</v>
+        <v>2717.8</v>
       </c>
       <c r="O24" s="2">
-        <v>3.9300000000000002E-2</v>
+        <v>4.8899999999999999E-2</v>
       </c>
       <c r="P24" s="2">
-        <v>4.1599999999999998E-2</v>
+        <v>5.6500000000000002E-2</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
@@ -4282,110 +4243,56 @@
         <v>46085</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality SMID Dividend Strategy (*SMID)</v>
       </c>
       <c r="C25" s="2">
-        <v>2.7300000000000001E-2</v>
+        <v>0.12130000000000001</v>
       </c>
       <c r="D25" t="str">
-        <f>"TROW"</f>
-        <v>TROW</v>
-      </c>
-      <c r="E25" t="str">
-        <f>"74144T108"</f>
-        <v>74144T108</v>
-      </c>
-      <c r="F25" t="str">
-        <f>"T. Rowe Price"</f>
-        <v>T. Rowe Price</v>
-      </c>
-      <c r="G25">
-        <v>756</v>
-      </c>
-      <c r="H25" s="1">
-        <v>45700</v>
-      </c>
-      <c r="I25" s="3">
-        <v>69544.44</v>
-      </c>
-      <c r="J25">
-        <v>91.99</v>
-      </c>
-      <c r="K25">
-        <v>106.27</v>
-      </c>
-      <c r="L25" s="3">
-        <v>80343.740000000005</v>
-      </c>
-      <c r="M25" s="3">
-        <v>3931.2</v>
-      </c>
-      <c r="N25" s="3">
-        <v>2717.8</v>
-      </c>
-      <c r="O25" s="2">
-        <v>4.8899999999999999E-2</v>
-      </c>
-      <c r="P25" s="2">
-        <v>5.6500000000000002E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B26" t="str">
-        <f>"*Quality SMID Dividend Strategy (*SMID)"</f>
-        <v>*Quality SMID Dividend Strategy (*SMID)</v>
-      </c>
-      <c r="C26" s="2">
-        <v>0.12130000000000001</v>
-      </c>
-      <c r="D26" t="str">
         <f>"CASH"</f>
         <v>CASH</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E25" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F26" t="str">
+      <c r="F25" t="str">
         <f>"Cash"</f>
         <v>Cash</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G25" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="H26" t="str">
+      <c r="H25" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="I26" s="3">
-        <v>309272.84000000003</v>
-      </c>
-      <c r="J26" t="str">
+      <c r="I25" s="3">
+        <v>349256.07</v>
+      </c>
+      <c r="J25" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="K26" t="str">
+      <c r="K25" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="L26" s="3">
-        <v>309272.84000000003</v>
-      </c>
-      <c r="M26" s="3">
+      <c r="L25" s="3">
+        <v>349256.07</v>
+      </c>
+      <c r="M25" s="3">
         <v>3092.73</v>
       </c>
-      <c r="N26">
+      <c r="N25">
         <v>0</v>
       </c>
-      <c r="O26" s="2">
+      <c r="O25" s="2">
         <v>0.01</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P25" s="2">
         <v>0.01</v>
       </c>
     </row>
@@ -4396,7 +4303,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C29E4F-58B6-4CCE-BC84-B1448CFC2599}">
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -4488,7 +4395,7 @@
         <v>46085</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" ref="B2:B47" si="0">"*Quality All-Cap Dividend Strategy (*DAC)"</f>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C2" s="2">
@@ -4542,7 +4449,7 @@
         <v>46085</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C3" s="2">
@@ -4596,7 +4503,7 @@
         <v>46085</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C4" s="2">
@@ -4650,7 +4557,7 @@
         <v>46085</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C5" s="2">
@@ -4704,7 +4611,7 @@
         <v>46085</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C6" s="2">
@@ -4758,7 +4665,7 @@
         <v>46085</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C7" s="2">
@@ -4811,7 +4718,7 @@
         <v>46085</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C8" s="2">
@@ -4865,7 +4772,7 @@
         <v>46085</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C9" s="2">
@@ -4918,7 +4825,7 @@
         <v>46085</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C10" s="2">
@@ -4972,7 +4879,7 @@
         <v>46085</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C11" s="2">
@@ -5025,7 +4932,7 @@
         <v>46085</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C12" s="2">
@@ -5079,7 +4986,7 @@
         <v>46085</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C13" s="2">
@@ -5132,7 +5039,7 @@
         <v>46085</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C14" s="2">
@@ -5186,7 +5093,7 @@
         <v>46085</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C15" s="2">
@@ -5240,7 +5147,7 @@
         <v>46085</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C16" s="2">
@@ -5293,7 +5200,7 @@
         <v>46085</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C17" s="2">
@@ -5346,7 +5253,7 @@
         <v>46085</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C18" s="2">
@@ -5399,7 +5306,7 @@
         <v>46085</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C19" s="2">
@@ -5452,7 +5359,7 @@
         <v>46085</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C20" s="2">
@@ -5505,7 +5412,7 @@
         <v>46085</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C21" s="2">
@@ -5558,7 +5465,7 @@
         <v>46085</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C22" s="2">
@@ -5611,7 +5518,7 @@
         <v>46085</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C23" s="2">
@@ -5665,7 +5572,7 @@
         <v>46085</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C24" s="2">
@@ -5718,7 +5625,7 @@
         <v>46085</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C25" s="2">
@@ -5736,7 +5643,7 @@
         <v>McCormick &amp; Co.</v>
       </c>
       <c r="G25">
-        <v>966</v>
+        <v>1311</v>
       </c>
       <c r="H25" s="1">
         <v>45980</v>
@@ -5771,7 +5678,7 @@
         <v>46085</v>
       </c>
       <c r="B26" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C26" s="2">
@@ -5825,7 +5732,7 @@
         <v>46085</v>
       </c>
       <c r="B27" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C27" s="2">
@@ -5878,7 +5785,7 @@
         <v>46085</v>
       </c>
       <c r="B28" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C28" s="2">
@@ -5931,7 +5838,7 @@
         <v>46085</v>
       </c>
       <c r="B29" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C29" s="2">
@@ -5984,7 +5891,7 @@
         <v>46085</v>
       </c>
       <c r="B30" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C30" s="2">
@@ -6037,7 +5944,7 @@
         <v>46085</v>
       </c>
       <c r="B31" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C31" s="2">
@@ -6090,7 +5997,7 @@
         <v>46085</v>
       </c>
       <c r="B32" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C32" s="2">
@@ -6143,7 +6050,7 @@
         <v>46085</v>
       </c>
       <c r="B33" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C33" s="2">
@@ -6196,7 +6103,7 @@
         <v>46085</v>
       </c>
       <c r="B34" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C34" s="2">
@@ -6249,7 +6156,7 @@
         <v>46085</v>
       </c>
       <c r="B35" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C35" s="2">
@@ -6303,7 +6210,7 @@
         <v>46085</v>
       </c>
       <c r="B36" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C36" s="2">
@@ -6356,7 +6263,7 @@
         <v>46085</v>
       </c>
       <c r="B37" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C37" s="2">
@@ -6410,7 +6317,7 @@
         <v>46085</v>
       </c>
       <c r="B38" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C38" s="2">
@@ -6463,7 +6370,7 @@
         <v>46085</v>
       </c>
       <c r="B39" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C39" s="2">
@@ -6516,52 +6423,52 @@
         <v>46085</v>
       </c>
       <c r="B40" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C40" s="2">
-        <v>7.1999999999999998E-3</v>
+        <v>1.2E-2</v>
       </c>
       <c r="D40" t="str">
-        <f>"RHI"</f>
-        <v>RHI</v>
+        <f>"SNA"</f>
+        <v>SNA</v>
       </c>
       <c r="E40">
-        <v>770323103</v>
+        <v>833034101</v>
       </c>
       <c r="F40" t="str">
-        <f>"Robert Half International"</f>
-        <v>Robert Half International</v>
+        <f>"Snap-On"</f>
+        <v>Snap-On</v>
       </c>
       <c r="G40">
-        <v>852</v>
+        <v>90</v>
       </c>
       <c r="H40" s="1">
-        <v>45470</v>
+        <v>43805</v>
       </c>
       <c r="I40" s="3">
-        <v>20720.64</v>
+        <v>34515</v>
       </c>
       <c r="J40">
-        <v>24.32</v>
+        <v>383.5</v>
       </c>
       <c r="K40">
-        <v>38.21</v>
+        <v>154.61000000000001</v>
       </c>
       <c r="L40" s="3">
-        <v>32558.240000000002</v>
-      </c>
-      <c r="M40" s="3">
-        <v>2010.72</v>
+        <v>13915.31</v>
+      </c>
+      <c r="M40">
+        <v>878.4</v>
       </c>
       <c r="N40" s="3">
-        <v>6529.91</v>
+        <v>4552.58</v>
       </c>
       <c r="O40" s="2">
-        <v>6.1800000000000001E-2</v>
+        <v>6.3100000000000003E-2</v>
       </c>
       <c r="P40" s="2">
-        <v>9.7000000000000003E-2</v>
+        <v>2.5399999999999999E-2</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
@@ -6569,52 +6476,52 @@
         <v>46085</v>
       </c>
       <c r="B41" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C41" s="2">
-        <v>1.2E-2</v>
+        <v>1.06E-2</v>
       </c>
       <c r="D41" t="str">
-        <f>"SNA"</f>
-        <v>SNA</v>
+        <f>"SWK"</f>
+        <v>SWK</v>
       </c>
       <c r="E41">
-        <v>833034101</v>
+        <v>854502101</v>
       </c>
       <c r="F41" t="str">
-        <f>"Snap-On"</f>
-        <v>Snap-On</v>
+        <f>"Stanley Black &amp; Decker"</f>
+        <v>Stanley Black &amp; Decker</v>
       </c>
       <c r="G41">
-        <v>90</v>
+        <v>381</v>
       </c>
       <c r="H41" s="1">
-        <v>43805</v>
+        <v>45442</v>
       </c>
       <c r="I41" s="3">
-        <v>34515</v>
+        <v>30396.18</v>
       </c>
       <c r="J41">
-        <v>383.5</v>
+        <v>79.78</v>
       </c>
       <c r="K41">
-        <v>154.61000000000001</v>
+        <v>84.36</v>
       </c>
       <c r="L41" s="3">
-        <v>13915.31</v>
-      </c>
-      <c r="M41">
-        <v>878.4</v>
+        <v>32141.07</v>
+      </c>
+      <c r="M41" s="3">
+        <v>1264.92</v>
       </c>
       <c r="N41" s="3">
-        <v>4552.58</v>
+        <v>1867.35</v>
       </c>
       <c r="O41" s="2">
-        <v>6.3100000000000003E-2</v>
+        <v>3.9399999999999998E-2</v>
       </c>
       <c r="P41" s="2">
-        <v>2.5399999999999999E-2</v>
+        <v>4.1599999999999998E-2</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
@@ -6622,52 +6529,53 @@
         <v>46085</v>
       </c>
       <c r="B42" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C42" s="2">
-        <v>1.06E-2</v>
+        <v>1.54E-2</v>
       </c>
       <c r="D42" t="str">
-        <f>"SWK"</f>
-        <v>SWK</v>
-      </c>
-      <c r="E42">
-        <v>854502101</v>
+        <f>"TROW"</f>
+        <v>TROW</v>
+      </c>
+      <c r="E42" t="str">
+        <f>"74144T108"</f>
+        <v>74144T108</v>
       </c>
       <c r="F42" t="str">
-        <f>"Stanley Black &amp; Decker"</f>
-        <v>Stanley Black &amp; Decker</v>
+        <f>"T. Rowe Price"</f>
+        <v>T. Rowe Price</v>
       </c>
       <c r="G42">
-        <v>381</v>
+        <v>480</v>
       </c>
       <c r="H42" s="1">
-        <v>45442</v>
+        <v>44929</v>
       </c>
       <c r="I42" s="3">
-        <v>30396.18</v>
+        <v>44155.199999999997</v>
       </c>
       <c r="J42">
-        <v>79.78</v>
+        <v>91.99</v>
       </c>
       <c r="K42">
-        <v>84.36</v>
+        <v>108.14</v>
       </c>
       <c r="L42" s="3">
-        <v>32141.07</v>
+        <v>51905.69</v>
       </c>
       <c r="M42" s="3">
-        <v>1264.92</v>
+        <v>2496</v>
       </c>
       <c r="N42" s="3">
-        <v>1867.35</v>
+        <v>6001.57</v>
       </c>
       <c r="O42" s="2">
-        <v>3.9399999999999998E-2</v>
+        <v>4.8099999999999997E-2</v>
       </c>
       <c r="P42" s="2">
-        <v>4.1599999999999998E-2</v>
+        <v>5.6500000000000002E-2</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
@@ -6675,53 +6583,52 @@
         <v>46085</v>
       </c>
       <c r="B43" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C43" s="2">
-        <v>1.54E-2</v>
+        <v>2.18E-2</v>
       </c>
       <c r="D43" t="str">
-        <f>"TROW"</f>
-        <v>TROW</v>
-      </c>
-      <c r="E43" t="str">
-        <f>"74144T108"</f>
-        <v>74144T108</v>
+        <f>"TXN"</f>
+        <v>TXN</v>
+      </c>
+      <c r="E43">
+        <v>882508104</v>
       </c>
       <c r="F43" t="str">
-        <f>"T. Rowe Price"</f>
-        <v>T. Rowe Price</v>
+        <f>"Texas Instruments"</f>
+        <v>Texas Instruments</v>
       </c>
       <c r="G43">
-        <v>480</v>
+        <v>310</v>
       </c>
       <c r="H43" s="1">
-        <v>44929</v>
+        <v>42369</v>
       </c>
       <c r="I43" s="3">
-        <v>44155.199999999997</v>
+        <v>62740.9</v>
       </c>
       <c r="J43">
-        <v>91.99</v>
+        <v>202.39</v>
       </c>
       <c r="K43">
-        <v>108.14</v>
+        <v>54.81</v>
       </c>
       <c r="L43" s="3">
-        <v>51905.69</v>
+        <v>16991.099999999999</v>
       </c>
       <c r="M43" s="3">
-        <v>2496</v>
+        <v>1760.8</v>
       </c>
       <c r="N43" s="3">
-        <v>6001.57</v>
+        <v>12220.2</v>
       </c>
       <c r="O43" s="2">
-        <v>4.8099999999999997E-2</v>
+        <v>0.1036</v>
       </c>
       <c r="P43" s="2">
-        <v>5.6500000000000002E-2</v>
+        <v>2.81E-2</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
@@ -6729,52 +6636,52 @@
         <v>46085</v>
       </c>
       <c r="B44" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C44" s="2">
-        <v>2.18E-2</v>
+        <v>2.1700000000000001E-2</v>
       </c>
       <c r="D44" t="str">
-        <f>"TXN"</f>
-        <v>TXN</v>
+        <f>"UNP"</f>
+        <v>UNP</v>
       </c>
       <c r="E44">
-        <v>882508104</v>
+        <v>907818108</v>
       </c>
       <c r="F44" t="str">
-        <f>"Texas Instruments"</f>
-        <v>Texas Instruments</v>
+        <f>"Union Pacific"</f>
+        <v>Union Pacific</v>
       </c>
       <c r="G44">
-        <v>310</v>
+        <v>234</v>
       </c>
       <c r="H44" s="1">
-        <v>42369</v>
+        <v>45092</v>
       </c>
       <c r="I44" s="3">
-        <v>62740.9</v>
+        <v>62407.8</v>
       </c>
       <c r="J44">
-        <v>202.39</v>
+        <v>266.7</v>
       </c>
       <c r="K44">
-        <v>54.81</v>
+        <v>213.43</v>
       </c>
       <c r="L44" s="3">
-        <v>16991.099999999999</v>
+        <v>49942.38</v>
       </c>
       <c r="M44" s="3">
-        <v>1760.8</v>
+        <v>1291.68</v>
       </c>
       <c r="N44" s="3">
-        <v>12220.2</v>
+        <v>2233.3200000000002</v>
       </c>
       <c r="O44" s="2">
-        <v>0.1036</v>
+        <v>2.5899999999999999E-2</v>
       </c>
       <c r="P44" s="2">
-        <v>2.81E-2</v>
+        <v>2.07E-2</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -6782,52 +6689,52 @@
         <v>46085</v>
       </c>
       <c r="B45" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C45" s="2">
-        <v>2.1700000000000001E-2</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="D45" t="str">
-        <f>"UNP"</f>
-        <v>UNP</v>
+        <f>"UPS"</f>
+        <v>UPS</v>
       </c>
       <c r="E45">
-        <v>907818108</v>
+        <v>911312106</v>
       </c>
       <c r="F45" t="str">
-        <f>"Union Pacific"</f>
-        <v>Union Pacific</v>
+        <f>"United Parcel Service"</f>
+        <v>United Parcel Service</v>
       </c>
       <c r="G45">
-        <v>234</v>
+        <v>482</v>
       </c>
       <c r="H45" s="1">
-        <v>45092</v>
+        <v>45470</v>
       </c>
       <c r="I45" s="3">
-        <v>62407.8</v>
+        <v>53261</v>
       </c>
       <c r="J45">
-        <v>266.7</v>
+        <v>110.5</v>
       </c>
       <c r="K45">
-        <v>213.43</v>
+        <v>101.08</v>
       </c>
       <c r="L45" s="3">
-        <v>49942.38</v>
+        <v>48721.21</v>
       </c>
       <c r="M45" s="3">
-        <v>1291.68</v>
+        <v>3161.92</v>
       </c>
       <c r="N45" s="3">
-        <v>2233.3200000000002</v>
+        <v>11659.65</v>
       </c>
       <c r="O45" s="2">
-        <v>2.5899999999999999E-2</v>
+        <v>6.4899999999999999E-2</v>
       </c>
       <c r="P45" s="2">
-        <v>2.07E-2</v>
+        <v>5.9400000000000001E-2</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
@@ -6835,52 +6742,53 @@
         <v>46085</v>
       </c>
       <c r="B46" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C46" s="2">
-        <v>1.8499999999999999E-2</v>
+        <v>1.6299999999999999E-2</v>
       </c>
       <c r="D46" t="str">
-        <f>"UPS"</f>
-        <v>UPS</v>
-      </c>
-      <c r="E46">
-        <v>911312106</v>
+        <f>"VZ"</f>
+        <v>VZ</v>
+      </c>
+      <c r="E46" t="str">
+        <f>"92343V104"</f>
+        <v>92343V104</v>
       </c>
       <c r="F46" t="str">
-        <f>"United Parcel Service"</f>
-        <v>United Parcel Service</v>
+        <f>"Verizon"</f>
+        <v>Verizon</v>
       </c>
       <c r="G46">
-        <v>482</v>
+        <v>918</v>
       </c>
       <c r="H46" s="1">
-        <v>45470</v>
+        <v>42369</v>
       </c>
       <c r="I46" s="3">
-        <v>53261</v>
+        <v>47001.599999999999</v>
       </c>
       <c r="J46">
-        <v>110.5</v>
+        <v>51.2</v>
       </c>
       <c r="K46">
-        <v>101.08</v>
+        <v>46.75</v>
       </c>
       <c r="L46" s="3">
-        <v>48721.21</v>
+        <v>42918.64</v>
       </c>
       <c r="M46" s="3">
-        <v>3161.92</v>
+        <v>2597.94</v>
       </c>
       <c r="N46" s="3">
-        <v>11659.65</v>
+        <v>24415.65</v>
       </c>
       <c r="O46" s="2">
-        <v>6.4899999999999999E-2</v>
+        <v>6.0499999999999998E-2</v>
       </c>
       <c r="P46" s="2">
-        <v>5.9400000000000001E-2</v>
+        <v>5.5300000000000002E-2</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
@@ -6888,110 +6796,56 @@
         <v>46085</v>
       </c>
       <c r="B47" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
+        <f t="shared" si="0"/>
         <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
       </c>
       <c r="C47" s="2">
-        <v>1.6299999999999999E-2</v>
+        <v>0.13469999999999999</v>
       </c>
       <c r="D47" t="str">
-        <f>"VZ"</f>
-        <v>VZ</v>
-      </c>
-      <c r="E47" t="str">
-        <f>"92343V104"</f>
-        <v>92343V104</v>
-      </c>
-      <c r="F47" t="str">
-        <f>"Verizon"</f>
-        <v>Verizon</v>
-      </c>
-      <c r="G47">
-        <v>918</v>
-      </c>
-      <c r="H47" s="1">
-        <v>42369</v>
-      </c>
-      <c r="I47" s="3">
-        <v>47001.599999999999</v>
-      </c>
-      <c r="J47">
-        <v>51.2</v>
-      </c>
-      <c r="K47">
-        <v>46.75</v>
-      </c>
-      <c r="L47" s="3">
-        <v>42918.64</v>
-      </c>
-      <c r="M47" s="3">
-        <v>2597.94</v>
-      </c>
-      <c r="N47" s="3">
-        <v>24415.65</v>
-      </c>
-      <c r="O47" s="2">
-        <v>6.0499999999999998E-2</v>
-      </c>
-      <c r="P47" s="2">
-        <v>5.5300000000000002E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B48" t="str">
-        <f>"*Quality All-Cap Dividend Strategy (*DAC)"</f>
-        <v>*Quality All-Cap Dividend Strategy (*DAC)</v>
-      </c>
-      <c r="C48" s="2">
-        <v>0.13469999999999999</v>
-      </c>
-      <c r="D48" t="str">
         <f>"CASH"</f>
         <v>CASH</v>
       </c>
-      <c r="E48" t="str">
+      <c r="E47" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F48" t="str">
+      <c r="F47" t="str">
         <f>"Cash"</f>
         <v>Cash</v>
       </c>
-      <c r="G48" t="str">
+      <c r="G47" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="H48" t="str">
+      <c r="H47" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="I48" s="3">
-        <v>387432.85</v>
-      </c>
-      <c r="J48" t="str">
+      <c r="I47" s="3">
+        <v>388807.05</v>
+      </c>
+      <c r="J47" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="K48" t="str">
+      <c r="K47" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="L48" s="3">
-        <v>387432.85</v>
-      </c>
-      <c r="M48" s="3">
+      <c r="L47" s="3">
+        <v>388807.05</v>
+      </c>
+      <c r="M47" s="3">
         <v>3874.33</v>
       </c>
-      <c r="N48">
+      <c r="N47">
         <v>0</v>
       </c>
-      <c r="O48" s="2">
+      <c r="O47" s="2">
         <v>0.01</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P47" s="2">
         <v>0.01</v>
       </c>
     </row>
@@ -7002,7 +6856,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E02FF74-771B-42A4-BECD-DEE097FBE4B1}">
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -7094,7 +6948,7 @@
         <v>46085</v>
       </c>
       <c r="B2" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" ref="B2:B37" si="0">"*Oregon Dividend Strategy (*QDGR)"</f>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C2" s="2">
@@ -7148,7 +7002,7 @@
         <v>46085</v>
       </c>
       <c r="B3" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C3" s="2">
@@ -7202,7 +7056,7 @@
         <v>46085</v>
       </c>
       <c r="B4" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C4" s="2">
@@ -7256,7 +7110,7 @@
         <v>46085</v>
       </c>
       <c r="B5" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C5" s="2">
@@ -7309,7 +7163,7 @@
         <v>46085</v>
       </c>
       <c r="B6" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C6" s="2">
@@ -7363,7 +7217,7 @@
         <v>46085</v>
       </c>
       <c r="B7" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C7" s="2">
@@ -7416,7 +7270,7 @@
         <v>46085</v>
       </c>
       <c r="B8" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C8" s="2">
@@ -7469,7 +7323,7 @@
         <v>46085</v>
       </c>
       <c r="B9" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C9" s="2">
@@ -7523,7 +7377,7 @@
         <v>46085</v>
       </c>
       <c r="B10" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C10" s="2">
@@ -7576,7 +7430,7 @@
         <v>46085</v>
       </c>
       <c r="B11" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C11" s="2">
@@ -7629,7 +7483,7 @@
         <v>46085</v>
       </c>
       <c r="B12" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C12" s="2">
@@ -7682,7 +7536,7 @@
         <v>46085</v>
       </c>
       <c r="B13" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C13" s="2">
@@ -7735,7 +7589,7 @@
         <v>46085</v>
       </c>
       <c r="B14" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C14" s="2">
@@ -7789,7 +7643,7 @@
         <v>46085</v>
       </c>
       <c r="B15" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C15" s="2">
@@ -7842,7 +7696,7 @@
         <v>46085</v>
       </c>
       <c r="B16" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C16" s="2">
@@ -7895,7 +7749,7 @@
         <v>46085</v>
       </c>
       <c r="B17" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C17" s="2">
@@ -7949,7 +7803,7 @@
         <v>46085</v>
       </c>
       <c r="B18" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C18" s="2">
@@ -8002,7 +7856,7 @@
         <v>46085</v>
       </c>
       <c r="B19" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C19" s="2">
@@ -8055,7 +7909,7 @@
         <v>46085</v>
       </c>
       <c r="B20" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C20" s="2">
@@ -8108,7 +7962,7 @@
         <v>46085</v>
       </c>
       <c r="B21" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C21" s="2">
@@ -8161,7 +8015,7 @@
         <v>46085</v>
       </c>
       <c r="B22" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C22" s="2">
@@ -8214,7 +8068,7 @@
         <v>46085</v>
       </c>
       <c r="B23" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C23" s="2">
@@ -8267,7 +8121,7 @@
         <v>46085</v>
       </c>
       <c r="B24" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C24" s="2">
@@ -8320,7 +8174,7 @@
         <v>46085</v>
       </c>
       <c r="B25" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C25" s="2">
@@ -8374,7 +8228,7 @@
         <v>46085</v>
       </c>
       <c r="B26" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C26" s="2">
@@ -8427,7 +8281,7 @@
         <v>46085</v>
       </c>
       <c r="B27" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C27" s="2">
@@ -8481,7 +8335,7 @@
         <v>46085</v>
       </c>
       <c r="B28" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C28" s="2">
@@ -8534,7 +8388,7 @@
         <v>46085</v>
       </c>
       <c r="B29" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C29" s="2">
@@ -8587,52 +8441,52 @@
         <v>46085</v>
       </c>
       <c r="B30" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C30" s="2">
-        <v>3.44E-2</v>
+        <v>1.89E-2</v>
       </c>
       <c r="D30" t="str">
-        <f>"RHI"</f>
-        <v>RHI</v>
+        <f>"SWK"</f>
+        <v>SWK</v>
       </c>
       <c r="E30">
-        <v>770323103</v>
+        <v>854502101</v>
       </c>
       <c r="F30" t="str">
-        <f>"Robert Half International"</f>
-        <v>Robert Half International</v>
-      </c>
-      <c r="G30" s="3">
-        <v>2988</v>
+        <f>"Stanley Black &amp; Decker"</f>
+        <v>Stanley Black &amp; Decker</v>
+      </c>
+      <c r="G30">
+        <v>500</v>
       </c>
       <c r="H30" s="1">
-        <v>43864</v>
+        <v>45442</v>
       </c>
       <c r="I30" s="3">
-        <v>72668.160000000003</v>
+        <v>39890</v>
       </c>
       <c r="J30">
-        <v>24.32</v>
+        <v>79.78</v>
       </c>
       <c r="K30">
-        <v>46.61</v>
+        <v>76.45</v>
       </c>
       <c r="L30" s="3">
-        <v>139276.10999999999</v>
+        <v>38222.839999999997</v>
       </c>
       <c r="M30" s="3">
-        <v>7051.68</v>
+        <v>1660</v>
       </c>
       <c r="N30" s="3">
-        <v>12141.36</v>
+        <v>2358.34</v>
       </c>
       <c r="O30" s="2">
-        <v>5.0599999999999999E-2</v>
+        <v>4.3400000000000001E-2</v>
       </c>
       <c r="P30" s="2">
-        <v>9.7000000000000003E-2</v>
+        <v>4.1599999999999998E-2</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
@@ -8640,52 +8494,53 @@
         <v>46085</v>
       </c>
       <c r="B31" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C31" s="2">
-        <v>1.89E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="D31" t="str">
-        <f>"SWK"</f>
-        <v>SWK</v>
-      </c>
-      <c r="E31">
-        <v>854502101</v>
+        <f>"TROW"</f>
+        <v>TROW</v>
+      </c>
+      <c r="E31" t="str">
+        <f>"74144T108"</f>
+        <v>74144T108</v>
       </c>
       <c r="F31" t="str">
-        <f>"Stanley Black &amp; Decker"</f>
-        <v>Stanley Black &amp; Decker</v>
+        <f>"T. Rowe Price"</f>
+        <v>T. Rowe Price</v>
       </c>
       <c r="G31">
-        <v>500</v>
+        <v>526</v>
       </c>
       <c r="H31" s="1">
-        <v>45442</v>
+        <v>44932</v>
       </c>
       <c r="I31" s="3">
-        <v>39890</v>
+        <v>48386.74</v>
       </c>
       <c r="J31">
-        <v>79.78</v>
+        <v>91.99</v>
       </c>
       <c r="K31">
-        <v>76.45</v>
+        <v>108.18</v>
       </c>
       <c r="L31" s="3">
-        <v>38222.839999999997</v>
+        <v>56901.07</v>
       </c>
       <c r="M31" s="3">
-        <v>1660</v>
+        <v>2735.2</v>
       </c>
       <c r="N31" s="3">
-        <v>2358.34</v>
+        <v>6221.64</v>
       </c>
       <c r="O31" s="2">
-        <v>4.3400000000000001E-2</v>
+        <v>4.8099999999999997E-2</v>
       </c>
       <c r="P31" s="2">
-        <v>4.1599999999999998E-2</v>
+        <v>5.6500000000000002E-2</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
@@ -8693,53 +8548,52 @@
         <v>46085</v>
       </c>
       <c r="B32" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C32" s="2">
-        <v>2.29E-2</v>
+        <v>2.3099999999999999E-2</v>
       </c>
       <c r="D32" t="str">
-        <f>"TROW"</f>
-        <v>TROW</v>
-      </c>
-      <c r="E32" t="str">
-        <f>"74144T108"</f>
-        <v>74144T108</v>
+        <f>"TXN"</f>
+        <v>TXN</v>
+      </c>
+      <c r="E32">
+        <v>882508104</v>
       </c>
       <c r="F32" t="str">
-        <f>"T. Rowe Price"</f>
-        <v>T. Rowe Price</v>
+        <f>"Texas Instruments"</f>
+        <v>Texas Instruments</v>
       </c>
       <c r="G32">
-        <v>526</v>
+        <v>241</v>
       </c>
       <c r="H32" s="1">
-        <v>44932</v>
+        <v>42954</v>
       </c>
       <c r="I32" s="3">
-        <v>48386.74</v>
+        <v>48775.99</v>
       </c>
       <c r="J32">
-        <v>91.99</v>
+        <v>202.39</v>
       </c>
       <c r="K32">
-        <v>108.18</v>
+        <v>105.46</v>
       </c>
       <c r="L32" s="3">
-        <v>56901.07</v>
+        <v>25416.41</v>
       </c>
       <c r="M32" s="3">
-        <v>2735.2</v>
+        <v>1368.88</v>
       </c>
       <c r="N32" s="3">
-        <v>6221.64</v>
+        <v>9505.7999999999993</v>
       </c>
       <c r="O32" s="2">
-        <v>4.8099999999999997E-2</v>
+        <v>5.3900000000000003E-2</v>
       </c>
       <c r="P32" s="2">
-        <v>5.6500000000000002E-2</v>
+        <v>2.81E-2</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
@@ -8747,52 +8601,52 @@
         <v>46085</v>
       </c>
       <c r="B33" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C33" s="2">
-        <v>2.3099999999999999E-2</v>
+        <v>2.7300000000000001E-2</v>
       </c>
       <c r="D33" t="str">
-        <f>"TXN"</f>
-        <v>TXN</v>
+        <f>"UL"</f>
+        <v>UL</v>
       </c>
       <c r="E33">
-        <v>882508104</v>
+        <v>904767803</v>
       </c>
       <c r="F33" t="str">
-        <f>"Texas Instruments"</f>
-        <v>Texas Instruments</v>
+        <f>"Unilever PLC"</f>
+        <v>Unilever PLC</v>
       </c>
       <c r="G33">
-        <v>241</v>
+        <v>834</v>
       </c>
       <c r="H33" s="1">
-        <v>42954</v>
+        <v>43892</v>
       </c>
       <c r="I33" s="3">
-        <v>48775.99</v>
+        <v>57604.38</v>
       </c>
       <c r="J33">
-        <v>202.39</v>
+        <v>69.069999999999993</v>
       </c>
       <c r="K33">
-        <v>105.46</v>
+        <v>63.23</v>
       </c>
       <c r="L33" s="3">
-        <v>25416.41</v>
+        <v>52736.98</v>
       </c>
       <c r="M33" s="3">
-        <v>1368.88</v>
+        <v>1915.93</v>
       </c>
       <c r="N33" s="3">
-        <v>9505.7999999999993</v>
+        <v>7034.38</v>
       </c>
       <c r="O33" s="2">
-        <v>5.3900000000000003E-2</v>
+        <v>3.6299999999999999E-2</v>
       </c>
       <c r="P33" s="2">
-        <v>2.81E-2</v>
+        <v>3.3300000000000003E-2</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
@@ -8800,52 +8654,52 @@
         <v>46085</v>
       </c>
       <c r="B34" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C34" s="2">
-        <v>2.7300000000000001E-2</v>
+        <v>2.01E-2</v>
       </c>
       <c r="D34" t="str">
-        <f>"UL"</f>
-        <v>UL</v>
+        <f>"UNP"</f>
+        <v>UNP</v>
       </c>
       <c r="E34">
-        <v>904767803</v>
+        <v>907818108</v>
       </c>
       <c r="F34" t="str">
-        <f>"Unilever PLC"</f>
-        <v>Unilever PLC</v>
+        <f>"Union Pacific"</f>
+        <v>Union Pacific</v>
       </c>
       <c r="G34">
-        <v>834</v>
+        <v>159</v>
       </c>
       <c r="H34" s="1">
-        <v>43892</v>
+        <v>45092</v>
       </c>
       <c r="I34" s="3">
-        <v>57604.38</v>
+        <v>42405.3</v>
       </c>
       <c r="J34">
-        <v>69.069999999999993</v>
+        <v>266.7</v>
       </c>
       <c r="K34">
-        <v>63.23</v>
+        <v>205.79</v>
       </c>
       <c r="L34" s="3">
-        <v>52736.98</v>
-      </c>
-      <c r="M34" s="3">
-        <v>1915.93</v>
+        <v>32721.08</v>
+      </c>
+      <c r="M34">
+        <v>877.68</v>
       </c>
       <c r="N34" s="3">
-        <v>7034.38</v>
+        <v>2330.94</v>
       </c>
       <c r="O34" s="2">
-        <v>3.6299999999999999E-2</v>
+        <v>2.6800000000000001E-2</v>
       </c>
       <c r="P34" s="2">
-        <v>3.3300000000000003E-2</v>
+        <v>2.07E-2</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
@@ -8853,52 +8707,52 @@
         <v>46085</v>
       </c>
       <c r="B35" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C35" s="2">
-        <v>2.01E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="D35" t="str">
-        <f>"UNP"</f>
-        <v>UNP</v>
+        <f>"UPS"</f>
+        <v>UPS</v>
       </c>
       <c r="E35">
-        <v>907818108</v>
+        <v>911312106</v>
       </c>
       <c r="F35" t="str">
-        <f>"Union Pacific"</f>
-        <v>Union Pacific</v>
+        <f>"United Parcel Service"</f>
+        <v>United Parcel Service</v>
       </c>
       <c r="G35">
-        <v>159</v>
+        <v>438</v>
       </c>
       <c r="H35" s="1">
-        <v>45092</v>
+        <v>43608</v>
       </c>
       <c r="I35" s="3">
-        <v>42405.3</v>
+        <v>48399</v>
       </c>
       <c r="J35">
-        <v>266.7</v>
+        <v>110.5</v>
       </c>
       <c r="K35">
-        <v>205.79</v>
+        <v>122.38</v>
       </c>
       <c r="L35" s="3">
-        <v>32721.08</v>
-      </c>
-      <c r="M35">
-        <v>877.68</v>
+        <v>53603.11</v>
+      </c>
+      <c r="M35" s="3">
+        <v>2873.28</v>
       </c>
       <c r="N35" s="3">
-        <v>2330.94</v>
+        <v>9887.61</v>
       </c>
       <c r="O35" s="2">
-        <v>2.6800000000000001E-2</v>
+        <v>5.3600000000000002E-2</v>
       </c>
       <c r="P35" s="2">
-        <v>2.07E-2</v>
+        <v>5.9400000000000001E-2</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
@@ -8906,52 +8760,53 @@
         <v>46085</v>
       </c>
       <c r="B36" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C36" s="2">
-        <v>2.29E-2</v>
+        <v>2.8199999999999999E-2</v>
       </c>
       <c r="D36" t="str">
-        <f>"UPS"</f>
-        <v>UPS</v>
-      </c>
-      <c r="E36">
-        <v>911312106</v>
+        <f>"VZ"</f>
+        <v>VZ</v>
+      </c>
+      <c r="E36" t="str">
+        <f>"92343V104"</f>
+        <v>92343V104</v>
       </c>
       <c r="F36" t="str">
-        <f>"United Parcel Service"</f>
-        <v>United Parcel Service</v>
-      </c>
-      <c r="G36">
-        <v>438</v>
+        <f>"Verizon"</f>
+        <v>Verizon</v>
+      </c>
+      <c r="G36" s="3">
+        <v>1163</v>
       </c>
       <c r="H36" s="1">
-        <v>43608</v>
+        <v>42954</v>
       </c>
       <c r="I36" s="3">
-        <v>48399</v>
+        <v>59545.599999999999</v>
       </c>
       <c r="J36">
-        <v>110.5</v>
+        <v>51.2</v>
       </c>
       <c r="K36">
-        <v>122.38</v>
+        <v>48.98</v>
       </c>
       <c r="L36" s="3">
-        <v>53603.11</v>
+        <v>56964.68</v>
       </c>
       <c r="M36" s="3">
-        <v>2873.28</v>
+        <v>3291.29</v>
       </c>
       <c r="N36" s="3">
-        <v>9887.61</v>
+        <v>18334</v>
       </c>
       <c r="O36" s="2">
-        <v>5.3600000000000002E-2</v>
+        <v>5.7799999999999997E-2</v>
       </c>
       <c r="P36" s="2">
-        <v>5.9400000000000001E-2</v>
+        <v>5.5300000000000002E-2</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
@@ -8959,110 +8814,56 @@
         <v>46085</v>
       </c>
       <c r="B37" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
+        <f t="shared" si="0"/>
         <v>*Oregon Dividend Strategy (*QDGR)</v>
       </c>
       <c r="C37" s="2">
-        <v>2.8199999999999999E-2</v>
+        <v>0.10970000000000001</v>
       </c>
       <c r="D37" t="str">
-        <f>"VZ"</f>
-        <v>VZ</v>
-      </c>
-      <c r="E37" t="str">
-        <f>"92343V104"</f>
-        <v>92343V104</v>
-      </c>
-      <c r="F37" t="str">
-        <f>"Verizon"</f>
-        <v>Verizon</v>
-      </c>
-      <c r="G37" s="3">
-        <v>1163</v>
-      </c>
-      <c r="H37" s="1">
-        <v>42954</v>
-      </c>
-      <c r="I37" s="3">
-        <v>59545.599999999999</v>
-      </c>
-      <c r="J37">
-        <v>51.2</v>
-      </c>
-      <c r="K37">
-        <v>48.98</v>
-      </c>
-      <c r="L37" s="3">
-        <v>56964.68</v>
-      </c>
-      <c r="M37" s="3">
-        <v>3291.29</v>
-      </c>
-      <c r="N37" s="3">
-        <v>18334</v>
-      </c>
-      <c r="O37" s="2">
-        <v>5.7799999999999997E-2</v>
-      </c>
-      <c r="P37" s="2">
-        <v>5.5300000000000002E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B38" t="str">
-        <f>"*Oregon Dividend Strategy (*QDGR)"</f>
-        <v>*Oregon Dividend Strategy (*QDGR)</v>
-      </c>
-      <c r="C38" s="2">
-        <v>0.10970000000000001</v>
-      </c>
-      <c r="D38" t="str">
         <f>"CASH"</f>
         <v>CASH</v>
       </c>
-      <c r="E38" t="str">
+      <c r="E37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F38" t="str">
+      <c r="F37" t="str">
         <f>"Cash"</f>
         <v>Cash</v>
       </c>
-      <c r="G38" t="str">
+      <c r="G37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="H38" t="str">
+      <c r="H37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="I38" s="3">
-        <v>231795.9</v>
-      </c>
-      <c r="J38" t="str">
+      <c r="I37" s="3">
+        <v>306928.93</v>
+      </c>
+      <c r="J37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="K38" t="str">
+      <c r="K37" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="L38" s="3">
-        <v>231795.9</v>
-      </c>
-      <c r="M38" s="3">
+      <c r="L37" s="3">
+        <v>306928.93</v>
+      </c>
+      <c r="M37" s="3">
         <v>2317.96</v>
       </c>
-      <c r="N38">
+      <c r="N37">
         <v>0</v>
       </c>
-      <c r="O38" s="2">
+      <c r="O37" s="2">
         <v>0.01</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P37" s="2">
         <v>0.01</v>
       </c>
     </row>
@@ -9073,7 +8874,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D84081D8-5611-4965-AEF8-EFCFA7E7E30B}">
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -10951,48 +10752,49 @@
         <v>0</v>
       </c>
       <c r="C36" s="2">
-        <v>4.3E-3</v>
+        <v>7.3499999999999996E-2</v>
       </c>
       <c r="D36" t="str">
-        <f>"RHI"</f>
-        <v>RHI</v>
-      </c>
-      <c r="E36">
-        <v>770323103</v>
+        <f>"XOP"</f>
+        <v>XOP</v>
+      </c>
+      <c r="E36" t="str">
+        <f>"78468R556"</f>
+        <v>78468R556</v>
       </c>
       <c r="F36" t="str">
-        <f>"Robert Half International"</f>
-        <v>Robert Half International</v>
+        <f>"SPDR® S&amp;P Oil &amp; Gas Explor &amp; Prodtn ETF"</f>
+        <v>SPDR® S&amp;P Oil &amp; Gas Explor &amp; Prodtn ETF</v>
       </c>
       <c r="G36">
-        <v>360</v>
+        <v>934</v>
       </c>
       <c r="H36" s="1">
-        <v>46024</v>
+        <v>45979</v>
       </c>
       <c r="I36" s="3">
-        <v>8755.2000000000007</v>
+        <v>150159.18</v>
       </c>
       <c r="J36">
-        <v>24.32</v>
+        <v>160.77000000000001</v>
       </c>
       <c r="K36">
-        <v>27.04</v>
+        <v>130.66</v>
       </c>
       <c r="L36" s="3">
-        <v>9732.6</v>
-      </c>
-      <c r="M36">
-        <v>849.6</v>
+        <v>122034.62</v>
+      </c>
+      <c r="M36" s="3">
+        <v>3086.82</v>
       </c>
       <c r="N36">
-        <v>0</v>
+        <v>486.14</v>
       </c>
       <c r="O36" s="2">
-        <v>8.7300000000000003E-2</v>
+        <v>2.53E-2</v>
       </c>
       <c r="P36" s="2">
-        <v>9.7000000000000003E-2</v>
+        <v>2.06E-2</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
@@ -11003,49 +10805,49 @@
         <v>0</v>
       </c>
       <c r="C37" s="2">
-        <v>7.3499999999999996E-2</v>
+        <v>7.9000000000000008E-3</v>
       </c>
       <c r="D37" t="str">
-        <f>"XOP"</f>
-        <v>XOP</v>
+        <f>"TROW"</f>
+        <v>TROW</v>
       </c>
       <c r="E37" t="str">
-        <f>"78468R556"</f>
-        <v>78468R556</v>
+        <f>"74144T108"</f>
+        <v>74144T108</v>
       </c>
       <c r="F37" t="str">
-        <f>"SPDR® S&amp;P Oil &amp; Gas Explor &amp; Prodtn ETF"</f>
-        <v>SPDR® S&amp;P Oil &amp; Gas Explor &amp; Prodtn ETF</v>
+        <f>"T. Rowe Price"</f>
+        <v>T. Rowe Price</v>
       </c>
       <c r="G37">
-        <v>934</v>
+        <v>175</v>
       </c>
       <c r="H37" s="1">
-        <v>45979</v>
+        <v>46024</v>
       </c>
       <c r="I37" s="3">
-        <v>150159.18</v>
+        <v>16098.25</v>
       </c>
       <c r="J37">
-        <v>160.77000000000001</v>
+        <v>91.99</v>
       </c>
       <c r="K37">
-        <v>130.66</v>
+        <v>102.93</v>
       </c>
       <c r="L37" s="3">
-        <v>122034.62</v>
-      </c>
-      <c r="M37" s="3">
-        <v>3086.82</v>
+        <v>18012.16</v>
+      </c>
+      <c r="M37">
+        <v>910</v>
       </c>
       <c r="N37">
-        <v>486.14</v>
+        <v>0</v>
       </c>
       <c r="O37" s="2">
-        <v>2.53E-2</v>
+        <v>5.0500000000000003E-2</v>
       </c>
       <c r="P37" s="2">
-        <v>2.06E-2</v>
+        <v>5.6500000000000002E-2</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
@@ -11056,49 +10858,48 @@
         <v>0</v>
       </c>
       <c r="C38" s="2">
-        <v>7.9000000000000008E-3</v>
+        <v>1.49E-2</v>
       </c>
       <c r="D38" t="str">
-        <f>"TROW"</f>
-        <v>TROW</v>
-      </c>
-      <c r="E38" t="str">
-        <f>"74144T108"</f>
-        <v>74144T108</v>
+        <f>"TXN"</f>
+        <v>TXN</v>
+      </c>
+      <c r="E38">
+        <v>882508104</v>
       </c>
       <c r="F38" t="str">
-        <f>"T. Rowe Price"</f>
-        <v>T. Rowe Price</v>
+        <f>"Texas Instruments"</f>
+        <v>Texas Instruments</v>
       </c>
       <c r="G38">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="H38" s="1">
-        <v>46024</v>
+        <v>41675</v>
       </c>
       <c r="I38" s="3">
-        <v>16098.25</v>
+        <v>30358.5</v>
       </c>
       <c r="J38">
-        <v>91.99</v>
+        <v>202.39</v>
       </c>
       <c r="K38">
-        <v>102.93</v>
+        <v>40.479999999999997</v>
       </c>
       <c r="L38" s="3">
-        <v>18012.16</v>
+        <v>6072.09</v>
       </c>
       <c r="M38">
-        <v>910</v>
-      </c>
-      <c r="N38">
-        <v>0</v>
+        <v>852</v>
+      </c>
+      <c r="N38" s="3">
+        <v>12793.4</v>
       </c>
       <c r="O38" s="2">
-        <v>5.0500000000000003E-2</v>
+        <v>0.14030000000000001</v>
       </c>
       <c r="P38" s="2">
-        <v>5.6500000000000002E-2</v>
+        <v>2.81E-2</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
@@ -11109,48 +10910,50 @@
         <v>0</v>
       </c>
       <c r="C39" s="2">
-        <v>1.49E-2</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="D39" t="str">
-        <f>"TXN"</f>
-        <v>TXN</v>
-      </c>
-      <c r="E39">
-        <v>882508104</v>
+        <f>"TTE"</f>
+        <v>TTE</v>
+      </c>
+      <c r="E39" t="str">
+        <f>"F92124100"</f>
+        <v>F92124100</v>
       </c>
       <c r="F39" t="str">
-        <f>"Texas Instruments"</f>
-        <v>Texas Instruments</v>
+        <f>"Total SA"</f>
+        <v>Total SA</v>
       </c>
       <c r="G39">
-        <v>150</v>
+        <v>259</v>
       </c>
       <c r="H39" s="1">
-        <v>41675</v>
+        <v>43874</v>
       </c>
       <c r="I39" s="3">
-        <v>30358.5</v>
+        <v>19922.28</v>
       </c>
       <c r="J39">
-        <v>202.39</v>
+        <v>76.92</v>
       </c>
       <c r="K39">
-        <v>40.479999999999997</v>
+        <v>49.35</v>
       </c>
       <c r="L39" s="3">
-        <v>6072.09</v>
+        <v>12782.93</v>
       </c>
       <c r="M39">
-        <v>852</v>
+        <v>0</v>
       </c>
       <c r="N39" s="3">
-        <v>12793.4</v>
-      </c>
-      <c r="O39" s="2">
-        <v>0.14030000000000001</v>
+        <v>9242.0499999999993</v>
+      </c>
+      <c r="O39" t="str">
+        <f>""</f>
+        <v/>
       </c>
       <c r="P39" s="2">
-        <v>2.81E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
@@ -11161,259 +10964,259 @@
         <v>0</v>
       </c>
       <c r="C40" s="2">
-        <v>9.7999999999999997E-3</v>
+        <v>1.4E-2</v>
       </c>
       <c r="D40" t="str">
-        <f>"TTE"</f>
-        <v>TTE</v>
-      </c>
-      <c r="E40" t="str">
-        <f>"F92124100"</f>
-        <v>F92124100</v>
+        <f>"UL"</f>
+        <v>UL</v>
+      </c>
+      <c r="E40">
+        <v>904767803</v>
       </c>
       <c r="F40" t="str">
-        <f>"Total SA"</f>
-        <v>Total SA</v>
+        <f>"Unilever PLC"</f>
+        <v>Unilever PLC</v>
       </c>
       <c r="G40">
-        <v>259</v>
+        <v>414</v>
       </c>
       <c r="H40" s="1">
-        <v>43874</v>
+        <v>43906</v>
       </c>
       <c r="I40" s="3">
-        <v>19922.28</v>
+        <v>28594.98</v>
       </c>
       <c r="J40">
-        <v>76.92</v>
+        <v>69.069999999999993</v>
       </c>
       <c r="K40">
-        <v>49.35</v>
+        <v>52.78</v>
       </c>
       <c r="L40" s="3">
-        <v>12782.93</v>
+        <v>21852.28</v>
       </c>
       <c r="M40">
+        <v>951.07</v>
+      </c>
+      <c r="N40" s="3">
+        <v>11509.06</v>
+      </c>
+      <c r="O40" s="2">
+        <v>4.3499999999999997E-2</v>
+      </c>
+      <c r="P40" s="2">
+        <v>3.3300000000000003E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B41" t="s">
         <v>0</v>
       </c>
-      <c r="N40" s="3">
-        <v>9242.0499999999993</v>
-      </c>
-      <c r="O40" t="str">
+      <c r="C41" s="2">
+        <v>7.1000000000000004E-3</v>
+      </c>
+      <c r="D41" t="str">
+        <f>"UNP"</f>
+        <v>UNP</v>
+      </c>
+      <c r="E41">
+        <v>907818108</v>
+      </c>
+      <c r="F41" t="str">
+        <f>"Union Pacific"</f>
+        <v>Union Pacific</v>
+      </c>
+      <c r="G41">
+        <v>54</v>
+      </c>
+      <c r="H41" s="1">
+        <v>45092</v>
+      </c>
+      <c r="I41" s="3">
+        <v>14401.8</v>
+      </c>
+      <c r="J41">
+        <v>266.7</v>
+      </c>
+      <c r="K41">
+        <v>205.84</v>
+      </c>
+      <c r="L41" s="3">
+        <v>11115.38</v>
+      </c>
+      <c r="M41">
+        <v>298.08</v>
+      </c>
+      <c r="N41" s="3">
+        <v>2044.62</v>
+      </c>
+      <c r="O41" s="2">
+        <v>2.6800000000000001E-2</v>
+      </c>
+      <c r="P41" s="2">
+        <v>2.07E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B42" t="s">
+        <v>0</v>
+      </c>
+      <c r="C42" s="2">
+        <v>1.04E-2</v>
+      </c>
+      <c r="D42" t="str">
+        <f>"UPS"</f>
+        <v>UPS</v>
+      </c>
+      <c r="E42">
+        <v>911312106</v>
+      </c>
+      <c r="F42" t="str">
+        <f>"United Parcel Service"</f>
+        <v>United Parcel Service</v>
+      </c>
+      <c r="G42">
+        <v>193</v>
+      </c>
+      <c r="H42" s="1">
+        <v>45924</v>
+      </c>
+      <c r="I42" s="3">
+        <v>21326.5</v>
+      </c>
+      <c r="J42">
+        <v>110.5</v>
+      </c>
+      <c r="K42">
+        <v>84.17</v>
+      </c>
+      <c r="L42" s="3">
+        <v>16245.2</v>
+      </c>
+      <c r="M42" s="3">
+        <v>1266.08</v>
+      </c>
+      <c r="N42" s="3">
+        <v>11683.6</v>
+      </c>
+      <c r="O42" s="2">
+        <v>7.7899999999999997E-2</v>
+      </c>
+      <c r="P42" s="2">
+        <v>5.9400000000000001E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B43" t="s">
+        <v>0</v>
+      </c>
+      <c r="C43" s="2">
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="D43" t="str">
+        <f>"VZ"</f>
+        <v>VZ</v>
+      </c>
+      <c r="E43" t="str">
+        <f>"92343V104"</f>
+        <v>92343V104</v>
+      </c>
+      <c r="F43" t="str">
+        <f>"Verizon"</f>
+        <v>Verizon</v>
+      </c>
+      <c r="G43">
+        <v>377</v>
+      </c>
+      <c r="H43" s="1">
+        <v>42241</v>
+      </c>
+      <c r="I43" s="3">
+        <v>19302.400000000001</v>
+      </c>
+      <c r="J43">
+        <v>51.2</v>
+      </c>
+      <c r="K43">
+        <v>36.86</v>
+      </c>
+      <c r="L43" s="3">
+        <v>13896.79</v>
+      </c>
+      <c r="M43" s="3">
+        <v>1066.9100000000001</v>
+      </c>
+      <c r="N43" s="3">
+        <v>25086.27</v>
+      </c>
+      <c r="O43" s="2">
+        <v>7.6799999999999993E-2</v>
+      </c>
+      <c r="P43" s="2">
+        <v>5.5300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B44" t="s">
+        <v>0</v>
+      </c>
+      <c r="C44" s="2">
+        <v>2.5399999999999999E-2</v>
+      </c>
+      <c r="D44" t="str">
+        <f>"CEF"</f>
+        <v>CEF</v>
+      </c>
+      <c r="E44" t="str">
+        <f>"85208R101"</f>
+        <v>85208R101</v>
+      </c>
+      <c r="F44" t="str">
+        <f>"Sprott Physical Gold and Silver Trust"</f>
+        <v>Sprott Physical Gold and Silver Trust</v>
+      </c>
+      <c r="G44">
+        <v>980</v>
+      </c>
+      <c r="H44" s="1">
+        <v>45979</v>
+      </c>
+      <c r="I44" s="3">
+        <v>51802.8</v>
+      </c>
+      <c r="J44">
+        <v>52.86</v>
+      </c>
+      <c r="K44">
+        <v>38.89</v>
+      </c>
+      <c r="L44" s="3">
+        <v>38109.06</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="P40" s="2">
+      <c r="P44" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B41" t="s">
-        <v>0</v>
-      </c>
-      <c r="C41" s="2">
-        <v>1.4E-2</v>
-      </c>
-      <c r="D41" t="str">
-        <f>"UL"</f>
-        <v>UL</v>
-      </c>
-      <c r="E41">
-        <v>904767803</v>
-      </c>
-      <c r="F41" t="str">
-        <f>"Unilever PLC"</f>
-        <v>Unilever PLC</v>
-      </c>
-      <c r="G41">
-        <v>414</v>
-      </c>
-      <c r="H41" s="1">
-        <v>43906</v>
-      </c>
-      <c r="I41" s="3">
-        <v>28594.98</v>
-      </c>
-      <c r="J41">
-        <v>69.069999999999993</v>
-      </c>
-      <c r="K41">
-        <v>52.78</v>
-      </c>
-      <c r="L41" s="3">
-        <v>21852.28</v>
-      </c>
-      <c r="M41">
-        <v>951.07</v>
-      </c>
-      <c r="N41" s="3">
-        <v>11509.06</v>
-      </c>
-      <c r="O41" s="2">
-        <v>4.3499999999999997E-2</v>
-      </c>
-      <c r="P41" s="2">
-        <v>3.3300000000000003E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B42" t="s">
-        <v>0</v>
-      </c>
-      <c r="C42" s="2">
-        <v>7.1000000000000004E-3</v>
-      </c>
-      <c r="D42" t="str">
-        <f>"UNP"</f>
-        <v>UNP</v>
-      </c>
-      <c r="E42">
-        <v>907818108</v>
-      </c>
-      <c r="F42" t="str">
-        <f>"Union Pacific"</f>
-        <v>Union Pacific</v>
-      </c>
-      <c r="G42">
-        <v>54</v>
-      </c>
-      <c r="H42" s="1">
-        <v>45092</v>
-      </c>
-      <c r="I42" s="3">
-        <v>14401.8</v>
-      </c>
-      <c r="J42">
-        <v>266.7</v>
-      </c>
-      <c r="K42">
-        <v>205.84</v>
-      </c>
-      <c r="L42" s="3">
-        <v>11115.38</v>
-      </c>
-      <c r="M42">
-        <v>298.08</v>
-      </c>
-      <c r="N42" s="3">
-        <v>2044.62</v>
-      </c>
-      <c r="O42" s="2">
-        <v>2.6800000000000001E-2</v>
-      </c>
-      <c r="P42" s="2">
-        <v>2.07E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B43" t="s">
-        <v>0</v>
-      </c>
-      <c r="C43" s="2">
-        <v>1.04E-2</v>
-      </c>
-      <c r="D43" t="str">
-        <f>"UPS"</f>
-        <v>UPS</v>
-      </c>
-      <c r="E43">
-        <v>911312106</v>
-      </c>
-      <c r="F43" t="str">
-        <f>"United Parcel Service"</f>
-        <v>United Parcel Service</v>
-      </c>
-      <c r="G43">
-        <v>193</v>
-      </c>
-      <c r="H43" s="1">
-        <v>45924</v>
-      </c>
-      <c r="I43" s="3">
-        <v>21326.5</v>
-      </c>
-      <c r="J43">
-        <v>110.5</v>
-      </c>
-      <c r="K43">
-        <v>84.17</v>
-      </c>
-      <c r="L43" s="3">
-        <v>16245.2</v>
-      </c>
-      <c r="M43" s="3">
-        <v>1266.08</v>
-      </c>
-      <c r="N43" s="3">
-        <v>11683.6</v>
-      </c>
-      <c r="O43" s="2">
-        <v>7.7899999999999997E-2</v>
-      </c>
-      <c r="P43" s="2">
-        <v>5.9400000000000001E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B44" t="s">
-        <v>0</v>
-      </c>
-      <c r="C44" s="2">
-        <v>9.4999999999999998E-3</v>
-      </c>
-      <c r="D44" t="str">
-        <f>"VZ"</f>
-        <v>VZ</v>
-      </c>
-      <c r="E44" t="str">
-        <f>"92343V104"</f>
-        <v>92343V104</v>
-      </c>
-      <c r="F44" t="str">
-        <f>"Verizon"</f>
-        <v>Verizon</v>
-      </c>
-      <c r="G44">
-        <v>377</v>
-      </c>
-      <c r="H44" s="1">
-        <v>42241</v>
-      </c>
-      <c r="I44" s="3">
-        <v>19302.400000000001</v>
-      </c>
-      <c r="J44">
-        <v>51.2</v>
-      </c>
-      <c r="K44">
-        <v>36.86</v>
-      </c>
-      <c r="L44" s="3">
-        <v>13896.79</v>
-      </c>
-      <c r="M44" s="3">
-        <v>1066.9100000000001</v>
-      </c>
-      <c r="N44" s="3">
-        <v>25086.27</v>
-      </c>
-      <c r="O44" s="2">
-        <v>7.6799999999999993E-2</v>
-      </c>
-      <c r="P44" s="2">
-        <v>5.5300000000000002E-2</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -11424,106 +11227,52 @@
         <v>0</v>
       </c>
       <c r="C45" s="2">
-        <v>2.5399999999999999E-2</v>
+        <v>3.3000000000000002E-2</v>
       </c>
       <c r="D45" t="str">
-        <f>"CEF"</f>
-        <v>CEF</v>
+        <f>"CASH"</f>
+        <v>CASH</v>
       </c>
       <c r="E45" t="str">
-        <f>"85208R101"</f>
-        <v>85208R101</v>
-      </c>
-      <c r="F45" t="str">
-        <f>"Sprott Physical Gold and Silver Trust"</f>
-        <v>Sprott Physical Gold and Silver Trust</v>
-      </c>
-      <c r="G45">
-        <v>980</v>
-      </c>
-      <c r="H45" s="1">
-        <v>45979</v>
-      </c>
-      <c r="I45" s="3">
-        <v>51802.8</v>
-      </c>
-      <c r="J45">
-        <v>52.86</v>
-      </c>
-      <c r="K45">
-        <v>38.89</v>
-      </c>
-      <c r="L45" s="3">
-        <v>38109.06</v>
-      </c>
-      <c r="M45">
-        <v>0</v>
-      </c>
-      <c r="N45">
-        <v>0</v>
-      </c>
-      <c r="O45" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="P45" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
-        <v>46085</v>
-      </c>
-      <c r="B46" t="s">
-        <v>0</v>
-      </c>
-      <c r="C46" s="2">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="D46" t="str">
-        <f>"CASH"</f>
-        <v>CASH</v>
-      </c>
-      <c r="E46" t="str">
+      <c r="F45" t="str">
+        <f>"Cash"</f>
+        <v>Cash</v>
+      </c>
+      <c r="G45" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F46" t="str">
-        <f>"Cash"</f>
-        <v>Cash</v>
-      </c>
-      <c r="G46" t="str">
+      <c r="H45" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="H46" t="str">
+      <c r="I45" s="3">
+        <v>67352.87</v>
+      </c>
+      <c r="J45" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="I46" s="3">
-        <v>67352.87</v>
-      </c>
-      <c r="J46" t="str">
+      <c r="K45" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="K46" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="L46" s="3">
+      <c r="L45" s="3">
         <v>67352.87</v>
       </c>
-      <c r="M46">
+      <c r="M45">
         <v>673.53</v>
       </c>
-      <c r="N46" s="3">
+      <c r="N45" s="3">
         <v>1956.82</v>
       </c>
-      <c r="O46" s="2">
+      <c r="O45" s="2">
         <v>0.01</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P45" s="2">
         <v>0.01</v>
       </c>
     </row>
@@ -11533,6 +11282,29 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -11745,37 +11517,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E299E2A-1D17-4E86-B664-ACAE02310EA4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00BBF7BA-55D0-4489-A50B-488CEE3798CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D43E81CF-20D7-4D83-A313-594A3398A52A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D43E81CF-20D7-4D83-A313-594A3398A52A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00BBF7BA-55D0-4489-A50B-488CEE3798CB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E299E2A-1D17-4E86-B664-ACAE02310EA4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-04-06 08:20
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -11176,4 +11176,252 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30EA02FA-659B-4A61-BCE6-3E3A9422C017}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA2E77B-7DE6-42EF-8EC9-6F7130597970}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09706853-4066-4EC6-A903-D42071203B64}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac 2026-04-17 10:42
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -11589,4 +11589,252 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B3478A9-DF88-4CDC-B3AF-DB4EF466FAFB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D224C83-A064-4723-AEC1-0BEE4895A364}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{207B0F5E-FDCB-46D4-ABF2-766F7FE3D101}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-21 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{913CC95C-6643-4E88-8475-4F994B30A047}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E710317F-9C8F-4E56-A971-3B0EFF96D43A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{244BD9CE-C786-490A-875B-269C22801E8D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-22 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22D67435-F597-42AC-BF1E-1F006072D70C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4546EE4-FD0C-456B-A95C-29A23AA0C112}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07D09247-6D7D-4589-A76A-EBCF11E019E8}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-25 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C827BFA6-4795-48B8-9869-756A1BBCB1D5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB6C42BA-DC8C-441A-9EED-B34B51B7A22C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{480660E3-0353-4C58-85A7-65420776E395}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-26 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2168945B-4B7D-47D6-9EB8-EC54EF18B791}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACEAD7FD-69CF-42F0-85AD-1F48407D9856}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89CBE816-F91A-4E18-92E2-67C8B282DA05}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-27 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4A2C0F-45E4-4C1F-948A-E76FADFF822F}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AFE5594E-9430-4D9E-97BA-C520E1680427}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C8974C3-8E63-451C-BBE9-B07F416245D8}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-28 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{934E1BAC-1565-46FA-A40A-EE8FF54271E5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4B85A26-6D93-45D1-8D62-F6DA1E898F3B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93C874DB-FA99-47CE-B8D8-57329E711ECB}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-05-29 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09B8A3B1-4F86-4BA5-890B-1694AB45D111}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98700763-BA1E-4032-9E02-F59589774C9E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE25714F-9796-4230-9E0A-CEA669C305EF}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings 2026-06-01 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B37BD925-7854-4989-877C-9F513C2002DB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80813644-15B8-4958-B87F-065A8A39C44A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D92153F0-AD2B-45BF-8986-EE87E73F863A}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-02 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7201,4 +7201,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{492C7381-544E-44C8-AAE0-41FDE365F9F5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{594992AF-2497-484C-95C8-003329ADD71A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{272FC3B6-0762-4ED7-A199-B561627E2B3F}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-03 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E14CADC-2451-4937-9B7C-801310BE430D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26CAC1C9-DC55-4773-9E0B-A31EE9EFDC52}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A81F0B56-C87C-4BD1-B577-5FF5B7DDCAE4}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-04 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04939FF9-CF76-476B-93D2-BF6AE29B12C2}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6FAC235-4C27-46B3-9BDB-6EC7EAA841E6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4ABA417-9A63-402C-AE82-4851CC45E233}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-05 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06C49601-EC20-4293-AD7C-1736727EB435}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D5F18E-A40F-4264-8920-9AF6FA05D03E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4BCB5FE-0D0A-4DD0-8971-666904DD84AF}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-08 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD626933-49F1-4D93-B2B0-5B3BCC4CF944}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D979152-C970-4A80-9474-C5F79BB46604}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A513C45-8F2F-4CBF-A4C0-3BB7839CFAB6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-09 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77B87A8A-6CBC-492A-BF4F-B81890D2567A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{889A55BF-62A7-448D-A7FD-997353012051}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6D5EDB8-2885-4F0D-B7E5-D8FE608A1AA6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-10 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F770F4AB-43E5-467A-BD15-CC30E2F8C547}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B383411F-303F-46E7-97BC-C8A240B78A05}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A00DB61-09F8-4290-9BB6-B7427331F4C2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-11 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7411,4 +7411,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61A74B09-32D4-4999-AD39-997FA2E14BE0}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40557544-6253-40E8-ACC4-618116BDCF74}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A15E197D-C5AB-4BD0-B00D-6517CB73E7E6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-12 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2B9EAF5-9893-4287-A027-CCA820990918}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4E88D6C-05CC-462F-908B-EB4D7BB22C71}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56914668-8C3A-42B5-88D6-388133061F93}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-15 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A8C0B1D-E40D-472C-953A-FA2AC421A4D7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2633BA4-0D0D-4BBB-9813-B583AA20CBB9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06216C76-B7E8-4AA0-A5B6-89776A5D0000}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-16 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{242FF0C2-1014-4CE9-AE20-1FFBFF253791}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC4E5831-CB00-41CB-87C1-ADD6D35E084E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{983777FA-15B5-45EE-A9C1-1BE45003B098}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-17 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0689BCE1-9597-478F-BC9B-7B9A076A261B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF8F0C55-0C99-4C0E-B077-D03A126FFDD4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B259E01-C552-45E1-9925-39DD1137721E}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-18 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2EC1EFC-56AF-4F3C-B178-E5944B146430}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3AB45AE-A41D-420D-BF94-76A12991A003}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5A8D4CF-55B3-42A6-BC19-6115893B2823}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-19 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48A96F93-58A3-4E5A-90E6-F81C50957698}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{562B6BAE-A4EF-489E-9680-201B7231944D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E6BC83A-AAA7-4C3E-9B57-03708D775624}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-22 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B48B7CF9-A3FB-4C94-8F08-4CAA7CE378B2}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84071818-DB84-48EA-B936-C800AFF10E77}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24D6EE8-2C11-4884-96EE-71A1CDF30ECC}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-23 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F1A89B1-54D9-47A2-8030-D6C5FDB443D1}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0823018-65D9-43F9-90AC-48C3548C2C36}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A80E5E45-A5FE-4BE5-898E-DF9261662B59}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-24 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F31B81B-4047-4C2B-95E5-0CA67913BACE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AF4B269-95FF-4753-A902-DE1128AF9B1B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F473ABB-3B39-469C-8897-2039DCDA7358}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-25 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45E24B7C-3D05-49A5-8C14-21FA6069F7F4}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD5FD229-60FD-416B-9EF8-C4AD63101B25}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCF5ACE1-F552-4A5F-A735-8EDA818C934D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-26 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7481,4 +7481,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21F2740D-B22B-401D-BEBF-53D9648BE3CB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{769E2633-D8E4-4BEE-B62E-B6A3B589E8B4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7E1F530-1BF0-4726-8247-14E7B98FD5C2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-29 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC6D76A3-4C3B-4B55-9CA9-987A5FCF5F8D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85D1A12A-E694-4640-9368-8E39B16E8616}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCF34EF1-3110-42DE-B2E7-4FD7CFE75F99}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-06-30 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E91CB2-4BD6-4A4E-A6E2-7FC8A1098C71}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAD6D22C-D02A-4C36-B9F2-E5FB8803A21C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C48AEA22-4282-469E-83A1-F9326B0D9E0F}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-01 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AAEE6C8-4D93-426B-AFE3-B181149D5EF9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC188CB4-DB87-4A6C-B902-050114C542A0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37519B50-57E3-4EF2-B9D6-E311BF00AB91}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-02 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D71E22F-67B7-4276-A171-8C7274E92585}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A131E38-5DB6-478E-86E1-3EFE90427C9F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79267793-5ABF-4C76-853A-3234908F80F5}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-03 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{820385B2-8D03-44A1-93C7-5025AD2B93BA}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{372E4F28-D69F-4D52-8291-85BCEB2532BD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F70D14E-69AD-4B2E-A5BE-726D312A3F13}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-06 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C206D283-5B7B-4AE7-B483-67CBB9F61C1C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CF2599F-C56F-4BBB-8F27-ABDFAC8E547E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CFA1030-991A-4982-BD26-465966F350D6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-07 06:33
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AE116E9-3298-498D-A2BE-5F4FE5C8FC23}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96C34111-BCD2-48DA-976A-9F0169A6444B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDF21EC7-1B81-4FDE-B2D7-4D8415CFBFDA}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-08 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A8FAE36-106D-4682-8C0E-39AEEC9772E5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A3104F25-0DE3-48D9-9C1E-D8857021E159}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22AF439A-B64F-493F-8DAA-80CA19CFD23D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-09 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3121E47B-6F83-4D83-A1F5-FC94DFA1B682}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{699CDA68-C4A6-448E-A632-2C68E393F999}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73851054-F844-40D7-9B93-F2826271D8EA}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-10 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABF431C9-EAF7-4A6D-A455-C722850F6E7A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD6D4804-2F3F-471E-B04B-C92C9B4804F0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221DC3BA-433B-46A6-8E82-64479A142742}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-13 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F736D643-D656-4D20-80A4-3FFA33B27685}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C0ACB61-9F9C-48A4-91E6-7566C33BCE56}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F535CA57-2318-49C0-ACAF-8E0DEC9B84FC}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-14 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA9BD602-B3CF-40DB-829C-F073081886E3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1F60B69-0714-416F-BBA1-627641D0E00D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557DADDB-3F11-4997-AC05-85EE0B0D44D2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-15 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D092D5F1-4573-4555-A16E-F72F501D44E3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACD924CB-C6F9-4A7A-9E07-0B6AF60BB42A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D9C6342-A275-469D-ADC8-88F84324E12B}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-16 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57DF38C0-4758-4767-B8A1-E050902F5090}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F69F2644-F372-4D55-96A6-C74DCBE1626F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68E8281E-7C70-4D89-BC39-94E719AD73E4}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-17 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{204A7BD4-5950-4E1E-B8EE-F0FC1F27CD4B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93961476-C5A5-4E59-9CEA-97BF03864BE9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C08B7CBE-056C-4CBF-9678-F8BFA2F8E3B3}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-20 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7642637C-55BF-4FB0-95A8-12638CEF20B6}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA1ECDDA-348A-4CC6-B3D9-EB7820484499}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03402819-DF74-4A2E-B324-A037FE9A968B}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-21 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B3C371D-B2EC-4CAF-8234-6A67FCE518D5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6B2E61C-DCE3-4B97-BC5C-B5D730AC50D9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77B84B06-39EB-4EB1-A581-41FFE7A80CC0}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-22 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32EDE5AD-FADB-4080-A58D-9B386677AC6E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F44CA8C-CA65-4E6E-AE08-29BA09A4FD44}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47C9FE90-81CB-44A8-B983-28258943420E}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-23 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FD9A183-77F4-4715-B8D5-9797589736AE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BEF3268-8EFD-4ED5-847C-BB8F28CE9BC8}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75B3DE06-92F8-425A-ABE3-053F22A3D32E}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-24 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA64E70F-A226-4A17-B126-E853CE75BB6B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E195ACB1-5D54-4604-91A8-F593E07196AD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01E68AEE-AE6C-4119-B968-1C4423D6923A}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-27 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29463001-FB1C-4E1C-8119-FA564DF5A9F0}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB238EDD-33D2-4D41-9639-DA525E449BFD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1E9CBDE-DFDA-40C5-965D-4EDACDCD5A02}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-28 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32C37922-21FA-42F8-930C-322A00FDD865}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C6623EE-80CB-4E65-B03A-90E6F67BD5EC}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D665C51-6D03-4C96-8D57-3AC1F0705508}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-29 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A2DA90-0969-4DFE-82AB-6B0689C3E87B}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2E386F6-7016-4C9C-856C-184202B87C24}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44C79BCA-6D3E-4A7F-A9C4-94F84A591427}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-30 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18056E8A-E1A9-4A84-A1FC-B68BF589AB27}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFE01118-E965-41ED-9C05-FB2F7BB65B77}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02D3ADE3-EC33-4C6C-92E0-E672E788972C}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-07-31 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E99D97B7-9AF3-430A-963B-6AF509C1577D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC64C6C2-D3F1-4874-A845-3F083CC5C1FE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49DF2F48-FDA4-451B-A225-061B0034F538}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-03 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66CD3067-1FE4-4527-A652-38A54E924E9D}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DFA0105-AD0D-4569-B4B9-6103FCBFEB42}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{752F56B8-3B5E-450B-88EB-EDD42D786794}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-04 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1429C8E9-BCEA-401C-8BF8-AAF89E262297}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3161FF44-575C-4928-850E-3143C8654D57}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A851E04-71E4-4F2D-929E-CCFE88E7C2BC}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-05 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DCD47D4-627C-4A23-BA33-1B6CC48D6E48}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5190163F-1DC6-404B-ABCD-B3B3E017A649}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9260FF49-A3FC-4CE7-B039-1490AE63EFB0}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-06 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FD05DDB-4A67-479E-AF80-CD750AB28F40}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10CB809C-F56A-41EE-B009-CFFA68890780}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{305A73F5-8904-42A3-BD16-65B8C1ABD606}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-07 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E6ED8BA-BD64-4481-B468-E737328D5FFB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30CBC111-AEE6-4B08-95E7-22C537EA4DBA}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C76CA578-6397-4821-8A5A-0ADF75C7553C}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-10 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A82AF90-0DE7-42CC-BA65-2012778A43D6}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4AF9A76-68A8-4BA8-A80F-11C1521DB44C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A977DB68-9DC4-4A4B-98F2-11E4D936EF6D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-11 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74AF843F-6E0E-41D2-89D8-60CA40668995}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC1688E1-3CC2-49C4-956C-D4136121D6AD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DDFA851-836E-4DFF-8C14-D68FE02AC585}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-12 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1874B06-CCFC-40A6-99C1-D7F12262136E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A1C376C-B97A-4785-BF05-B7200154D3AF}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C562E45-F26A-41D3-9736-B683A3EBED5D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-13 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04F8DB9D-664A-4BB1-8951-404C5461E88E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA917C0C-03EA-43D8-BFDD-8A3EA3BCCC0E}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DAA95D3-0938-46AC-A3B3-56AF3557D3E5}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-14 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FCC49D2-9032-4AC6-A15E-25FCF7248B66}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A54A264-7CB8-4B9B-9B6B-7FCC45F6A231}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AE02472-7029-45E0-AFE2-B4FD6436EBF4}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-17 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD275DE6-D03D-4797-9320-41F39853B138}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9361B78D-D1BE-4832-B8B9-36E97523F066}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{244DB9D6-FBDA-42A1-8812-305299DB5111}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-18 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A726A736-CFA9-4937-9F26-D8E56FC552F4}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1ED4A12-21FA-42F5-A010-5F76EB9A3499}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E33C490C-DA85-4E35-B9A7-93AF0E584AA4}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-19 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F3D88F8-2FFE-43AA-841A-283320A5B691}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4151C975-4C73-4C39-81F0-314EE6EFFF77}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{835EDD42-B9A8-4A07-A7F8-AE625FE57CD3}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-20 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD4779F0-440E-4995-981C-329B4FA95B7C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4800EA2-E8CB-4FB0-8A69-980E43FDFFB1}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C862DA7-B61D-4DD0-A726-92943855C4A6}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-21 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5BE2C2B-4FDB-4F05-A424-B7B4F410EEB6}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{178B00B0-B0DF-4EC7-9DBC-C42C28B87991}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B956B90-FDC6-4DED-84B6-945A7594F38F}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-24 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84A17F-F54D-48EA-AC22-D68FA79C37F8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C19CBA1A-6374-42BA-90D2-A6F193FF2057}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F5E999-36D1-41CD-878A-C24DBC8D59C2}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-26 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{906967C7-C130-4ED7-815F-9043FC1186FE}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3C8124F-DD3F-4E7E-8742-1A0894E18D51}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18498E62-6994-4814-A030-7B165CE45373}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-27 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7551,4 +7551,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50E52E35-5DFD-4989-B7DE-6B46E76B8499}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31C38F8B-497C-4CC5-B39F-0C161DFC07FC}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CCAEE7C-3F50-4992-A8E5-3BF5CF2E0B5B}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-28 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CC389A1-D4B1-4F67-9DE0-6C0232E55E97}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F8FAFC5-D169-4E17-A5B2-B9C363E746E9}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9BF74DE-3A34-4623-8384-AAE49F3FBF98}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-08-31 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD98DBFC-A8D9-4AB2-A178-B4868DE998B4}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E5BA6D-7407-486B-9FD8-EA853A29EDC6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E8E39F2-3AF6-4C5E-9300-49FB32FECC50}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-01 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C5BB33C-E149-478E-85A0-571BB7EF5E65}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6668FCDC-6995-4E91-B6F3-8A7D1F18ACAF}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A27479BD-A7D0-4FD7-B1EC-85BD3B987C2C}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-02 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FDB2D0B-3119-4F69-BAF6-B0FEA144372A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B9152A-D1C0-4FED-8088-5358ACF08D35}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07EA2385-C6B9-4FC6-B8B1-44FECFDD9FB1}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-03 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21E27128-6BE2-4D2F-B1CE-59FD2157D7D3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F910D4E-2DA3-4C99-833E-EAC20E18C6AE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E920FE7-870B-4F62-8433-FC1988399A02}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-04 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58B0D3A9-7202-48CB-B8E7-9F2F91B686F7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CD326AA-CFD9-4873-AFA9-D5F72889AD89}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B155F1A2-111E-4AF1-AE25-C14771316E7D}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-07 06:32
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF93F096-F9C2-4888-AE8A-C64A4DE8E8D0}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A2EEE56-1FD3-4F89-9A34-52DA782D6CC2}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{694CD800-D607-4E0C-8BF6-D87969327868}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-08 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF497E38-694C-490C-BF06-C10EF840AB87}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB5F258D-A652-4193-91B7-5B939AF4336D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F4D843D-64DB-4F6F-A999-BA33C7D5C80E}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-09 06:30
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2AD8135-F5B2-4ED8-A399-A48CE19B0C54}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6186E503-6D60-4CDB-8BFF-0E909011EC17}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6AE79B4-C798-401F-8D6D-A7F3CD35D2DF}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-10 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89F9E98B-0C1F-40D7-9502-08C6E3AFA397}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF6F253-F58E-49E3-A76A-CEF2177A234A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BC80D0A-4E88-4B0C-B067-ADF318991C52}"/>
 </file>
</xml_diff>

<commit_message>
Update Tamarac holdings (Tamarac_Holdings.xlsx) 2026-09-11 06:31
</commit_message>
<xml_diff>
--- a/data/Tamarac_Holdings.xlsx
+++ b/data/Tamarac_Holdings.xlsx
@@ -7621,4 +7621,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
+    <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <xsd:import namespace="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MigrationWizId" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdPermissions" minOccurs="0"/>
+                <xsd:element ref="ns2:MigrationWizIdVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db58b361-de72-439a-9b19-5afb42a4fe9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MigrationWizId" ma:index="8" nillable="true" ma:displayName="MigrationWizId" ma:internalName="MigrationWizId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdPermissions" ma:index="9" nillable="true" ma:displayName="MigrationWizIdPermissions" ma:internalName="MigrationWizIdPermissions">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MigrationWizIdVersion" ma:index="10" nillable="true" ma:displayName="MigrationWizIdVersion" ma:internalName="MigrationWizIdVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="96639c25-1a56-4197-b479-8befda008741" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e26837be-2e64-4fb1-8d10-81cb111b0084" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b3bc2a0c-107b-4c5c-910e-cb5bd0310dcf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e26837be-2e64-4fb1-8d10-81cb111b0084">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66747FDD-EF11-48DE-8659-FB96CD58A8C7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DBEAED-2D17-4D75-906D-38A31D57452D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7106B705-CA5D-4C1B-B85C-274E088BEB5B}"/>
 </file>
</xml_diff>